<commit_message>
Fix workbook showing blank cells in non-recalculating viewers
openpyxl wrote formulas with empty cached values (<v/>), so any app that
doesn't auto-recalc (Google Sheets import quirks, Numbers, mobile/preview,
Excel manual-calc) showed blank outputs. Injected 573 computed cached
values into formula cells while keeping formulas live. Verified: XML
well-formed, opens cleanly, displays numbers without recalc, and still
recalculates when inputs change.

https://claude.ai/code/session_01AV7mTHPnESeU9WjC2R7zG6
</commit_message>
<xml_diff>
--- a/castellan_btm_model/Castellan_BESS_Model.xlsx
+++ b/castellan_btm_model/Castellan_BESS_Model.xlsx
@@ -1568,7 +1568,7 @@
       </c>
       <c r="E12" s="37">
         <f>'Sizing Comparison'!J7</f>
-        <v/>
+        <v>6168.008</v>
       </c>
     </row>
     <row r="13">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="E13" s="37">
         <f>'Sizing Comparison'!M7</f>
-        <v/>
+        <v>80500</v>
       </c>
     </row>
     <row r="14">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="E14" s="38">
         <f>'Sizing Comparison'!N7</f>
-        <v/>
+        <v>13.05121524</v>
       </c>
     </row>
     <row r="15">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="E15" s="37">
         <f>'Sizing Comparison'!O7</f>
-        <v/>
+        <v>-45301.89769</v>
       </c>
     </row>
     <row r="16">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="E16" s="39">
         <f>'Sizing Comparison'!P7</f>
-        <v/>
+        <v>-0.035832867</v>
       </c>
     </row>
     <row r="17">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="E17" s="38">
         <f>'Value Stacking'!B17</f>
-        <v/>
+        <v>13.05121524</v>
       </c>
     </row>
     <row r="19">
@@ -1817,22 +1817,22 @@
       </c>
       <c r="B5" s="31">
         <f>'CF_Calc'!E7</f>
-        <v/>
+        <v>-80500</v>
       </c>
       <c r="C5" s="31">
         <f>B5</f>
-        <v/>
+        <v>-80500</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="31">
         <f>'CF_Calc'!E10</f>
-        <v/>
+        <v>-147000</v>
       </c>
       <c r="G5" s="31">
         <f>F5</f>
-        <v/>
+        <v>-147000</v>
       </c>
     </row>
     <row r="6">
@@ -1841,22 +1841,22 @@
       </c>
       <c r="B6" s="31">
         <f>'CF_Calc'!F7</f>
-        <v/>
+        <v>4443.008</v>
       </c>
       <c r="C6" s="31">
         <f>C5+B6</f>
-        <v/>
+        <v>-76056.992</v>
       </c>
       <c r="E6" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="31">
         <f>'CF_Calc'!F10</f>
-        <v/>
+        <v>4235.072</v>
       </c>
       <c r="G6" s="31">
         <f>G5+F6</f>
-        <v/>
+        <v>-142764.928</v>
       </c>
     </row>
     <row r="7">
@@ -1865,22 +1865,22 @@
       </c>
       <c r="B7" s="31">
         <f>'CF_Calc'!G7</f>
-        <v/>
+        <v>4404.652995</v>
       </c>
       <c r="C7" s="31">
         <f>C6+B7</f>
-        <v/>
+        <v>-71652.33901</v>
       </c>
       <c r="E7" t="n">
         <v>2</v>
       </c>
       <c r="F7" s="31">
         <f>'CF_Calc'!G10</f>
-        <v/>
+        <v>4167.45633</v>
       </c>
       <c r="G7" s="31">
         <f>G6+F7</f>
-        <v/>
+        <v>-138597.4717</v>
       </c>
     </row>
     <row r="8">
@@ -1889,22 +1889,22 @@
       </c>
       <c r="B8" s="31">
         <f>'CF_Calc'!H7</f>
-        <v/>
+        <v>4361.560235</v>
       </c>
       <c r="C8" s="31">
         <f>C7+B8</f>
-        <v/>
+        <v>-67290.77877</v>
       </c>
       <c r="E8" t="n">
         <v>3</v>
       </c>
       <c r="F8" s="31">
         <f>'CF_Calc'!H10</f>
-        <v/>
+        <v>4093.734206</v>
       </c>
       <c r="G8" s="31">
         <f>G7+F8</f>
-        <v/>
+        <v>-134503.7375</v>
       </c>
     </row>
     <row r="9">
@@ -1913,22 +1913,22 @@
       </c>
       <c r="B9" s="31">
         <f>'CF_Calc'!I7</f>
-        <v/>
+        <v>4313.515941</v>
       </c>
       <c r="C9" s="31">
         <f>C8+B9</f>
-        <v/>
+        <v>-62977.26283</v>
       </c>
       <c r="E9" t="n">
         <v>4</v>
       </c>
       <c r="F9" s="31">
         <f>'CF_Calc'!I10</f>
-        <v/>
+        <v>4013.640992</v>
       </c>
       <c r="G9" s="31">
         <f>G8+F9</f>
-        <v/>
+        <v>-130490.0965</v>
       </c>
     </row>
     <row r="10">
@@ -1937,22 +1937,22 @@
       </c>
       <c r="B10" s="31">
         <f>'CF_Calc'!J7</f>
-        <v/>
+        <v>4260.29859</v>
       </c>
       <c r="C10" s="31">
         <f>C9+B10</f>
-        <v/>
+        <v>-58716.96424</v>
       </c>
       <c r="E10" t="n">
         <v>5</v>
       </c>
       <c r="F10" s="31">
         <f>'CF_Calc'!J10</f>
-        <v/>
+        <v>3926.902601</v>
       </c>
       <c r="G10" s="31">
         <f>G9+F10</f>
-        <v/>
+        <v>-126563.1939</v>
       </c>
     </row>
     <row r="11">
@@ -1961,22 +1961,22 @@
       </c>
       <c r="B11" s="31">
         <f>'CF_Calc'!K7</f>
-        <v/>
+        <v>4201.678659</v>
       </c>
       <c r="C11" s="31">
         <f>C10+B11</f>
-        <v/>
+        <v>-54515.28558</v>
       </c>
       <c r="E11" t="n">
         <v>6</v>
       </c>
       <c r="F11" s="31">
         <f>'CF_Calc'!K10</f>
-        <v/>
+        <v>3833.235194</v>
       </c>
       <c r="G11" s="31">
         <f>G10+F11</f>
-        <v/>
+        <v>-122729.9587</v>
       </c>
     </row>
     <row r="12">
@@ -1985,22 +1985,22 @@
       </c>
       <c r="B12" s="31">
         <f>'CF_Calc'!L7</f>
-        <v/>
+        <v>4137.418366</v>
       </c>
       <c r="C12" s="31">
         <f>C11+B12</f>
-        <v/>
+        <v>-50377.86721</v>
       </c>
       <c r="E12" t="n">
         <v>7</v>
       </c>
       <c r="F12" s="31">
         <f>'CF_Calc'!L10</f>
-        <v/>
+        <v>3732.344862</v>
       </c>
       <c r="G12" s="31">
         <f>G11+F12</f>
-        <v/>
+        <v>-118997.6138</v>
       </c>
     </row>
     <row r="13">
@@ -2009,22 +2009,22 @@
       </c>
       <c r="B13" s="31">
         <f>'CF_Calc'!M7</f>
-        <v/>
+        <v>4067.271395</v>
       </c>
       <c r="C13" s="31">
         <f>C12+B13</f>
-        <v/>
+        <v>-46310.59582</v>
       </c>
       <c r="E13" t="n">
         <v>8</v>
       </c>
       <c r="F13" s="31">
         <f>'CF_Calc'!M10</f>
-        <v/>
+        <v>3623.927295</v>
       </c>
       <c r="G13" s="31">
         <f>G12+F13</f>
-        <v/>
+        <v>-115373.6865</v>
       </c>
     </row>
     <row r="14">
@@ -2033,22 +2033,22 @@
       </c>
       <c r="B14" s="31">
         <f>'CF_Calc'!N7</f>
-        <v/>
+        <v>3990.982623</v>
       </c>
       <c r="C14" s="31">
         <f>C13+B14</f>
-        <v/>
+        <v>-42319.6132</v>
       </c>
       <c r="E14" t="n">
         <v>9</v>
       </c>
       <c r="F14" s="31">
         <f>'CF_Calc'!N10</f>
-        <v/>
+        <v>3507.667448</v>
       </c>
       <c r="G14" s="31">
         <f>G13+F14</f>
-        <v/>
+        <v>-111866.0191</v>
       </c>
     </row>
     <row r="15">
@@ -2057,22 +2057,22 @@
       </c>
       <c r="B15" s="31">
         <f>'CF_Calc'!O7</f>
-        <v/>
+        <v>3908.287831</v>
       </c>
       <c r="C15" s="31">
         <f>C14+B15</f>
-        <v/>
+        <v>-38411.32537</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
       </c>
       <c r="F15" s="31">
         <f>'CF_Calc'!O10</f>
-        <v/>
+        <v>3383.239196</v>
       </c>
       <c r="G15" s="31">
         <f>G14+F15</f>
-        <v/>
+        <v>-108482.7799</v>
       </c>
     </row>
     <row r="16">
@@ -2081,22 +2081,22 @@
       </c>
       <c r="B16" s="31">
         <f>'CF_Calc'!P7</f>
-        <v/>
+        <v>3818.913407</v>
       </c>
       <c r="C16" s="31">
         <f>C15+B16</f>
-        <v/>
+        <v>-34592.41196</v>
       </c>
       <c r="E16" t="n">
         <v>11</v>
       </c>
       <c r="F16" s="31">
         <f>'CF_Calc'!P10</f>
-        <v/>
+        <v>3250.304971</v>
       </c>
       <c r="G16" s="31">
         <f>G15+F16</f>
-        <v/>
+        <v>-105232.4749</v>
       </c>
     </row>
     <row r="17">
@@ -2105,22 +2105,22 @@
       </c>
       <c r="B17" s="31">
         <f>'CF_Calc'!Q7</f>
-        <v/>
+        <v>3722.576044</v>
       </c>
       <c r="C17" s="31">
         <f>C16+B17</f>
-        <v/>
+        <v>-30869.83591</v>
       </c>
       <c r="E17" t="n">
         <v>12</v>
       </c>
       <c r="F17" s="31">
         <f>'CF_Calc'!Q10</f>
-        <v/>
+        <v>3108.515396</v>
       </c>
       <c r="G17" s="31">
         <f>G16+F17</f>
-        <v/>
+        <v>-102123.9595</v>
       </c>
     </row>
     <row r="18">
@@ -2129,22 +2129,22 @@
       </c>
       <c r="B18" s="31">
         <f>'CF_Calc'!R7</f>
-        <v/>
+        <v>3618.982423</v>
       </c>
       <c r="C18" s="31">
         <f>C17+B18</f>
-        <v/>
+        <v>-27250.85349</v>
       </c>
       <c r="E18" t="n">
         <v>13</v>
       </c>
       <c r="F18" s="31">
         <f>'CF_Calc'!R10</f>
-        <v/>
+        <v>2957.508906</v>
       </c>
       <c r="G18" s="31">
         <f>G17+F18</f>
-        <v/>
+        <v>-99166.4506</v>
       </c>
     </row>
     <row r="19">
@@ -2153,22 +2153,22 @@
       </c>
       <c r="B19" s="31">
         <f>'CF_Calc'!S7</f>
-        <v/>
+        <v>3507.828891</v>
       </c>
       <c r="C19" s="31">
         <f>C18+B19</f>
-        <v/>
+        <v>-23743.0246</v>
       </c>
       <c r="E19" t="n">
         <v>14</v>
       </c>
       <c r="F19" s="31">
         <f>'CF_Calc'!S10</f>
-        <v/>
+        <v>2796.911354</v>
       </c>
       <c r="G19" s="31">
         <f>G18+F19</f>
-        <v/>
+        <v>-96369.53925</v>
       </c>
     </row>
     <row r="20">
@@ -2177,22 +2177,22 @@
       </c>
       <c r="B20" s="31">
         <f>'CF_Calc'!T7</f>
-        <v/>
+        <v>3388.801124</v>
       </c>
       <c r="C20" s="31">
         <f>C19+B20</f>
-        <v/>
+        <v>-20354.22348</v>
       </c>
       <c r="E20" t="n">
         <v>15</v>
       </c>
       <c r="F20" s="31">
         <f>'CF_Calc'!T10</f>
-        <v/>
+        <v>2626.335608</v>
       </c>
       <c r="G20" s="31">
         <f>G19+F20</f>
-        <v/>
+        <v>-93743.20364</v>
       </c>
     </row>
     <row r="22">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="B22" s="32">
         <f>'Sizing Comparison'!N7</f>
-        <v/>
+        <v>13.05121524</v>
       </c>
       <c r="E22" s="30" t="inlineStr">
         <is>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="F22" s="32">
         <f>'Sizing Comparison'!N10</f>
-        <v/>
+        <v>19.90501921</v>
       </c>
     </row>
     <row r="23">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="B23" s="31">
         <f>'CF_Calc'!U7</f>
-        <v/>
+        <v>-45301.89769</v>
       </c>
       <c r="E23" s="30" t="inlineStr">
         <is>
@@ -2232,7 +2232,7 @@
       </c>
       <c r="F23" s="31">
         <f>'CF_Calc'!U10</f>
-        <v/>
+        <v>-115264.1005</v>
       </c>
     </row>
     <row r="24">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B24" s="33">
         <f>'CF_Calc'!V7</f>
-        <v/>
+        <v>-0.035832867</v>
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="F24" s="33">
         <f>'CF_Calc'!V10</f>
-        <v/>
+        <v>-0.1128356093</v>
       </c>
     </row>
   </sheetData>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="B13" s="12">
         <f>Assumptions!B24</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="B14" s="12">
         <f>'Sizing Comparison'!A7</f>
-        <v/>
+        <v>50</v>
       </c>
     </row>
     <row r="15">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="B15" s="14">
         <f>Assumptions!B25</f>
-        <v/>
+        <v>120</v>
       </c>
     </row>
     <row r="16">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="B16" s="43">
         <f>'Sizing Comparison'!G7</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2465,23 +2465,23 @@
       </c>
       <c r="B5" s="13">
         <f>(150*400*(1-Assumptions!$B$20))/(238.7*10)</f>
-        <v/>
+        <v>17.59530792</v>
       </c>
       <c r="C5" s="13">
         <f>(150*500*(1-Assumptions!$B$20))/(238.7*10)</f>
-        <v/>
+        <v>21.9941349</v>
       </c>
       <c r="D5" s="13">
         <f>(150*600*(1-Assumptions!$B$20))/(238.7*10)</f>
-        <v/>
+        <v>26.39296188</v>
       </c>
       <c r="E5" s="13">
         <f>(150*700*(1-Assumptions!$B$20))/(238.7*10)</f>
-        <v/>
+        <v>30.79178886</v>
       </c>
       <c r="F5" s="13">
         <f>(150*800*(1-Assumptions!$B$20))/(238.7*10)</f>
-        <v/>
+        <v>35.19061584</v>
       </c>
     </row>
     <row r="6">
@@ -2490,23 +2490,23 @@
       </c>
       <c r="B6" s="13">
         <f>(150*400*(1-Assumptions!$B$20))/(238.7*15)</f>
-        <v/>
+        <v>11.73020528</v>
       </c>
       <c r="C6" s="13">
         <f>(150*500*(1-Assumptions!$B$20))/(238.7*15)</f>
-        <v/>
+        <v>14.6627566</v>
       </c>
       <c r="D6" s="13">
         <f>(150*600*(1-Assumptions!$B$20))/(238.7*15)</f>
-        <v/>
+        <v>17.59530792</v>
       </c>
       <c r="E6" s="13">
         <f>(150*700*(1-Assumptions!$B$20))/(238.7*15)</f>
-        <v/>
+        <v>20.52785924</v>
       </c>
       <c r="F6" s="13">
         <f>(150*800*(1-Assumptions!$B$20))/(238.7*15)</f>
-        <v/>
+        <v>23.46041056</v>
       </c>
     </row>
     <row r="7">
@@ -2515,23 +2515,23 @@
       </c>
       <c r="B7" s="13">
         <f>(150*400*(1-Assumptions!$B$20))/(238.7*20)</f>
-        <v/>
+        <v>8.797653959</v>
       </c>
       <c r="C7" s="13">
         <f>(150*500*(1-Assumptions!$B$20))/(238.7*20)</f>
-        <v/>
+        <v>10.99706745</v>
       </c>
       <c r="D7" s="13">
         <f>(150*600*(1-Assumptions!$B$20))/(238.7*20)</f>
-        <v/>
+        <v>13.19648094</v>
       </c>
       <c r="E7" s="13">
         <f>(150*700*(1-Assumptions!$B$20))/(238.7*20)</f>
-        <v/>
+        <v>15.39589443</v>
       </c>
       <c r="F7" s="13">
         <f>(150*800*(1-Assumptions!$B$20))/(238.7*20)</f>
-        <v/>
+        <v>17.59530792</v>
       </c>
     </row>
     <row r="8">
@@ -2540,23 +2540,23 @@
       </c>
       <c r="B8" s="13">
         <f>(150*400*(1-Assumptions!$B$20))/(238.7*25.84)</f>
-        <v/>
+        <v>6.80932969</v>
       </c>
       <c r="C8" s="13">
         <f>(150*500*(1-Assumptions!$B$20))/(238.7*25.84)</f>
-        <v/>
+        <v>8.511662112</v>
       </c>
       <c r="D8" s="13">
         <f>(150*600*(1-Assumptions!$B$20))/(238.7*25.84)</f>
-        <v/>
+        <v>10.21399453</v>
       </c>
       <c r="E8" s="13">
         <f>(150*700*(1-Assumptions!$B$20))/(238.7*25.84)</f>
-        <v/>
+        <v>11.91632696</v>
       </c>
       <c r="F8" s="13">
         <f>(150*800*(1-Assumptions!$B$20))/(238.7*25.84)</f>
-        <v/>
+        <v>13.61865938</v>
       </c>
     </row>
     <row r="9">
@@ -2565,23 +2565,23 @@
       </c>
       <c r="B9" s="13">
         <f>(150*400*(1-Assumptions!$B$20))/(238.7*30)</f>
-        <v/>
+        <v>5.865102639</v>
       </c>
       <c r="C9" s="13">
         <f>(150*500*(1-Assumptions!$B$20))/(238.7*30)</f>
-        <v/>
+        <v>7.331378299</v>
       </c>
       <c r="D9" s="13">
         <f>(150*600*(1-Assumptions!$B$20))/(238.7*30)</f>
-        <v/>
+        <v>8.797653959</v>
       </c>
       <c r="E9" s="13">
         <f>(150*700*(1-Assumptions!$B$20))/(238.7*30)</f>
-        <v/>
+        <v>10.26392962</v>
       </c>
       <c r="F9" s="13">
         <f>(150*800*(1-Assumptions!$B$20))/(238.7*30)</f>
-        <v/>
+        <v>11.73020528</v>
       </c>
     </row>
     <row r="10">
@@ -2590,23 +2590,23 @@
       </c>
       <c r="B10" s="13">
         <f>(150*400*(1-Assumptions!$B$20))/(238.7*40)</f>
-        <v/>
+        <v>4.398826979</v>
       </c>
       <c r="C10" s="13">
         <f>(150*500*(1-Assumptions!$B$20))/(238.7*40)</f>
-        <v/>
+        <v>5.498533724</v>
       </c>
       <c r="D10" s="13">
         <f>(150*600*(1-Assumptions!$B$20))/(238.7*40)</f>
-        <v/>
+        <v>6.598240469</v>
       </c>
       <c r="E10" s="13">
         <f>(150*700*(1-Assumptions!$B$20))/(238.7*40)</f>
-        <v/>
+        <v>7.697947214</v>
       </c>
       <c r="F10" s="13">
         <f>(150*800*(1-Assumptions!$B$20))/(238.7*40)</f>
-        <v/>
+        <v>8.797653959</v>
       </c>
     </row>
     <row r="12">
@@ -3188,58 +3188,58 @@
       </c>
       <c r="C5" s="13">
         <f>B5/A5</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="D5" s="13" t="n">
         <v>153.9</v>
       </c>
       <c r="E5" s="14">
         <f>D5*Assumptions!$B$5</f>
-        <v/>
+        <v>3976.776</v>
       </c>
       <c r="F5" s="14">
         <f>B5*Assumptions!$B$13*Assumptions!$B$8*Assumptions!$B$9*Assumptions!$B$12</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G5" s="14">
         <f>A5*Assumptions!$B$25*Assumptions!$B$24</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H5" s="14">
         <f>A5*Assumptions!$B$28*Assumptions!$B$29</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I5" s="14">
         <f>Assumptions!$B$41</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J5" s="14">
         <f>E5+F5+G5+H5+I5</f>
-        <v/>
+        <v>3976.776</v>
       </c>
       <c r="K5" s="14">
         <f>A5*Assumptions!$B$17+B5*Assumptions!$B$18+Assumptions!$B$19</f>
-        <v/>
+        <v>62000</v>
       </c>
       <c r="L5" s="14">
         <f>K5*Assumptions!$B$20</f>
-        <v/>
+        <v>18600</v>
       </c>
       <c r="M5" s="14">
         <f>K5-L5-Assumptions!$B$21</f>
-        <v/>
+        <v>43400</v>
       </c>
       <c r="N5" s="13">
         <f>M5/J5</f>
-        <v/>
+        <v>10.91336299</v>
       </c>
       <c r="O5" s="14">
         <f>'CF_Calc'!U5</f>
-        <v/>
+        <v>-18958.1907</v>
       </c>
       <c r="P5" s="15">
         <f>'CF_Calc'!V5</f>
-        <v/>
+        <v>-0.004440704189</v>
       </c>
     </row>
     <row r="6">
@@ -3251,58 +3251,58 @@
       </c>
       <c r="C6" s="17">
         <f>B6/A6</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="D6" s="17" t="n">
         <v>199.7</v>
       </c>
       <c r="E6" s="18">
         <f>D6*Assumptions!$B$5</f>
-        <v/>
+        <v>5160.248</v>
       </c>
       <c r="F6" s="18">
         <f>B6*Assumptions!$B$13*Assumptions!$B$8*Assumptions!$B$9*Assumptions!$B$12</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G6" s="18">
         <f>A6*Assumptions!$B$25*Assumptions!$B$24</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H6" s="18">
         <f>A6*Assumptions!$B$28*Assumptions!$B$29</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I6" s="18">
         <f>Assumptions!$B$41</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J6" s="18">
         <f>E6+F6+G6+H6+I6</f>
-        <v/>
+        <v>5160.248</v>
       </c>
       <c r="K6" s="18">
         <f>A6*Assumptions!$B$17+B6*Assumptions!$B$18+Assumptions!$B$19</f>
-        <v/>
+        <v>90000</v>
       </c>
       <c r="L6" s="18">
         <f>K6*Assumptions!$B$20</f>
-        <v/>
+        <v>27000</v>
       </c>
       <c r="M6" s="18">
         <f>K6-L6-Assumptions!$B$21</f>
-        <v/>
+        <v>63000</v>
       </c>
       <c r="N6" s="17">
         <f>M6/J6</f>
-        <v/>
+        <v>12.20871555</v>
       </c>
       <c r="O6" s="18">
         <f>'CF_Calc'!U6</f>
-        <v/>
+        <v>-32658.82052</v>
       </c>
       <c r="P6" s="19">
         <f>'CF_Calc'!V6</f>
-        <v/>
+        <v>-0.02416452145</v>
       </c>
     </row>
     <row r="7">
@@ -3314,58 +3314,58 @@
       </c>
       <c r="C7" s="21">
         <f>B7/A7</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="D7" s="21" t="n">
         <v>238.7</v>
       </c>
       <c r="E7" s="22">
         <f>D7*Assumptions!$B$5</f>
-        <v/>
+        <v>6168.008</v>
       </c>
       <c r="F7" s="22">
         <f>B7*Assumptions!$B$13*Assumptions!$B$8*Assumptions!$B$9*Assumptions!$B$12</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G7" s="22">
         <f>A7*Assumptions!$B$25*Assumptions!$B$24</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H7" s="22">
         <f>A7*Assumptions!$B$28*Assumptions!$B$29</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I7" s="22">
         <f>Assumptions!$B$41</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J7" s="22">
         <f>E7+F7+G7+H7+I7</f>
-        <v/>
+        <v>6168.008</v>
       </c>
       <c r="K7" s="22">
         <f>A7*Assumptions!$B$17+B7*Assumptions!$B$18+Assumptions!$B$19</f>
-        <v/>
+        <v>115000</v>
       </c>
       <c r="L7" s="22">
         <f>K7*Assumptions!$B$20</f>
-        <v/>
+        <v>34500</v>
       </c>
       <c r="M7" s="22">
         <f>K7-L7-Assumptions!$B$21</f>
-        <v/>
+        <v>80500</v>
       </c>
       <c r="N7" s="21">
         <f>M7/J7</f>
-        <v/>
+        <v>13.05121524</v>
       </c>
       <c r="O7" s="22">
         <f>'CF_Calc'!U7</f>
-        <v/>
+        <v>-45301.89769</v>
       </c>
       <c r="P7" s="23">
         <f>'CF_Calc'!V7</f>
-        <v/>
+        <v>-0.035832867</v>
       </c>
     </row>
     <row r="8">
@@ -3377,58 +3377,58 @@
       </c>
       <c r="C8" s="17">
         <f>B8/A8</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="D8" s="17" t="n">
         <v>238.7</v>
       </c>
       <c r="E8" s="18">
         <f>D8*Assumptions!$B$5</f>
-        <v/>
+        <v>6168.008</v>
       </c>
       <c r="F8" s="18">
         <f>B8*Assumptions!$B$13*Assumptions!$B$8*Assumptions!$B$9*Assumptions!$B$12</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G8" s="18">
         <f>A8*Assumptions!$B$25*Assumptions!$B$24</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H8" s="18">
         <f>A8*Assumptions!$B$28*Assumptions!$B$29</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I8" s="18">
         <f>Assumptions!$B$41</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J8" s="18">
         <f>E8+F8+G8+H8+I8</f>
-        <v/>
+        <v>6168.008</v>
       </c>
       <c r="K8" s="18">
         <f>A8*Assumptions!$B$17+B8*Assumptions!$B$18+Assumptions!$B$19</f>
-        <v/>
+        <v>125000</v>
       </c>
       <c r="L8" s="18">
         <f>K8*Assumptions!$B$20</f>
-        <v/>
+        <v>37500</v>
       </c>
       <c r="M8" s="18">
         <f>K8-L8-Assumptions!$B$21</f>
-        <v/>
+        <v>87500</v>
       </c>
       <c r="N8" s="17">
         <f>M8/J8</f>
-        <v/>
+        <v>14.18610352</v>
       </c>
       <c r="O8" s="18">
         <f>'CF_Calc'!U8</f>
-        <v/>
+        <v>-53741.21312</v>
       </c>
       <c r="P8" s="19">
         <f>'CF_Calc'!V8</f>
-        <v/>
+        <v>-0.05043723692</v>
       </c>
     </row>
     <row r="9">
@@ -3440,58 +3440,58 @@
       </c>
       <c r="C9" s="13">
         <f>B9/A9</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="D9" s="13" t="n">
         <v>261</v>
       </c>
       <c r="E9" s="14">
         <f>D9*Assumptions!$B$5</f>
-        <v/>
+        <v>6744.24</v>
       </c>
       <c r="F9" s="14">
         <f>B9*Assumptions!$B$13*Assumptions!$B$8*Assumptions!$B$9*Assumptions!$B$12</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G9" s="14">
         <f>A9*Assumptions!$B$25*Assumptions!$B$24</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H9" s="14">
         <f>A9*Assumptions!$B$28*Assumptions!$B$29</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I9" s="14">
         <f>Assumptions!$B$41</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J9" s="14">
         <f>E9+F9+G9+H9+I9</f>
-        <v/>
+        <v>6744.24</v>
       </c>
       <c r="K9" s="14">
         <f>A9*Assumptions!$B$17+B9*Assumptions!$B$18+Assumptions!$B$19</f>
-        <v/>
+        <v>160000</v>
       </c>
       <c r="L9" s="14">
         <f>K9*Assumptions!$B$20</f>
-        <v/>
+        <v>48000</v>
       </c>
       <c r="M9" s="14">
         <f>K9-L9-Assumptions!$B$21</f>
-        <v/>
+        <v>112000</v>
       </c>
       <c r="N9" s="13">
         <f>M9/J9</f>
-        <v/>
+        <v>16.6067637</v>
       </c>
       <c r="O9" s="14">
         <f>'CF_Calc'!U9</f>
-        <v/>
+        <v>-78444.1706</v>
       </c>
       <c r="P9" s="15">
         <f>'CF_Calc'!V9</f>
-        <v/>
+        <v>-0.07851302868</v>
       </c>
     </row>
     <row r="10">
@@ -3503,58 +3503,58 @@
       </c>
       <c r="C10" s="17">
         <f>B10/A10</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="D10" s="17" t="n">
         <v>285.8</v>
       </c>
       <c r="E10" s="18">
         <f>D10*Assumptions!$B$5</f>
-        <v/>
+        <v>7385.072</v>
       </c>
       <c r="F10" s="18">
         <f>B10*Assumptions!$B$13*Assumptions!$B$8*Assumptions!$B$9*Assumptions!$B$12</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G10" s="18">
         <f>A10*Assumptions!$B$25*Assumptions!$B$24</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H10" s="18">
         <f>A10*Assumptions!$B$28*Assumptions!$B$29</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I10" s="18">
         <f>Assumptions!$B$41</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J10" s="18">
         <f>E10+F10+G10+H10+I10</f>
-        <v/>
+        <v>7385.072</v>
       </c>
       <c r="K10" s="18">
         <f>A10*Assumptions!$B$17+B10*Assumptions!$B$18+Assumptions!$B$19</f>
-        <v/>
+        <v>210000</v>
       </c>
       <c r="L10" s="18">
         <f>K10*Assumptions!$B$20</f>
-        <v/>
+        <v>63000</v>
       </c>
       <c r="M10" s="18">
         <f>K10-L10-Assumptions!$B$21</f>
-        <v/>
+        <v>147000</v>
       </c>
       <c r="N10" s="17">
         <f>M10/J10</f>
-        <v/>
+        <v>19.90501921</v>
       </c>
       <c r="O10" s="18">
         <f>'CF_Calc'!U10</f>
-        <v/>
+        <v>-115264.1005</v>
       </c>
       <c r="P10" s="19">
         <f>'CF_Calc'!V10</f>
-        <v/>
+        <v>-0.1128356093</v>
       </c>
     </row>
     <row r="11">
@@ -3566,58 +3566,58 @@
       </c>
       <c r="C11" s="13">
         <f>B11/A11</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="D11" s="13" t="n">
         <v>301.2</v>
       </c>
       <c r="E11" s="14">
         <f>D11*Assumptions!$B$5</f>
-        <v/>
+        <v>7783.008</v>
       </c>
       <c r="F11" s="14">
         <f>B11*Assumptions!$B$13*Assumptions!$B$8*Assumptions!$B$9*Assumptions!$B$12</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G11" s="14">
         <f>A11*Assumptions!$B$25*Assumptions!$B$24</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H11" s="14">
         <f>A11*Assumptions!$B$28*Assumptions!$B$29</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I11" s="14">
         <f>Assumptions!$B$41</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J11" s="14">
         <f>E11+F11+G11+H11+I11</f>
-        <v/>
+        <v>7783.008</v>
       </c>
       <c r="K11" s="14">
         <f>A11*Assumptions!$B$17+B11*Assumptions!$B$18+Assumptions!$B$19</f>
-        <v/>
+        <v>260000</v>
       </c>
       <c r="L11" s="14">
         <f>K11*Assumptions!$B$20</f>
-        <v/>
+        <v>78000</v>
       </c>
       <c r="M11" s="14">
         <f>K11-L11-Assumptions!$B$21</f>
-        <v/>
+        <v>182000</v>
       </c>
       <c r="N11" s="13">
         <f>M11/J11</f>
-        <v/>
+        <v>23.38427508</v>
       </c>
       <c r="O11" s="14">
         <f>'CF_Calc'!U11</f>
-        <v/>
+        <v>-154121.9531</v>
       </c>
       <c r="P11" s="15">
         <f>'CF_Calc'!V11</f>
-        <v/>
+        <v>-0.1475420424</v>
       </c>
     </row>
     <row r="12">
@@ -3629,58 +3629,58 @@
       </c>
       <c r="C12" s="17">
         <f>B12/A12</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="D12" s="17" t="n">
         <v>285.8</v>
       </c>
       <c r="E12" s="18">
         <f>D12*Assumptions!$B$5</f>
-        <v/>
+        <v>7385.072</v>
       </c>
       <c r="F12" s="18">
         <f>B12*Assumptions!$B$13*Assumptions!$B$8*Assumptions!$B$9*Assumptions!$B$12</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G12" s="18">
         <f>A12*Assumptions!$B$25*Assumptions!$B$24</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H12" s="18">
         <f>A12*Assumptions!$B$28*Assumptions!$B$29</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I12" s="18">
         <f>Assumptions!$B$41</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J12" s="18">
         <f>E12+F12+G12+H12+I12</f>
-        <v/>
+        <v>7385.072</v>
       </c>
       <c r="K12" s="18">
         <f>A12*Assumptions!$B$17+B12*Assumptions!$B$18+Assumptions!$B$19</f>
-        <v/>
+        <v>230000</v>
       </c>
       <c r="L12" s="18">
         <f>K12*Assumptions!$B$20</f>
-        <v/>
+        <v>69000</v>
       </c>
       <c r="M12" s="18">
         <f>K12-L12-Assumptions!$B$21</f>
-        <v/>
+        <v>161000</v>
       </c>
       <c r="N12" s="17">
         <f>M12/J12</f>
-        <v/>
+        <v>21.80073532</v>
       </c>
       <c r="O12" s="18">
         <f>'CF_Calc'!U12</f>
-        <v/>
+        <v>-132142.7313</v>
       </c>
       <c r="P12" s="19">
         <f>'CF_Calc'!V12</f>
-        <v/>
+        <v>-0.131715269</v>
       </c>
     </row>
     <row r="13">
@@ -3692,58 +3692,58 @@
       </c>
       <c r="C13" s="13">
         <f>B13/A13</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="D13" s="13" t="n">
         <v>301.2</v>
       </c>
       <c r="E13" s="14">
         <f>D13*Assumptions!$B$5</f>
-        <v/>
+        <v>7783.008</v>
       </c>
       <c r="F13" s="14">
         <f>B13*Assumptions!$B$13*Assumptions!$B$8*Assumptions!$B$9*Assumptions!$B$12</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G13" s="14">
         <f>A13*Assumptions!$B$25*Assumptions!$B$24</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H13" s="14">
         <f>A13*Assumptions!$B$28*Assumptions!$B$29</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I13" s="14">
         <f>Assumptions!$B$41</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J13" s="14">
         <f>E13+F13+G13+H13+I13</f>
-        <v/>
+        <v>7783.008</v>
       </c>
       <c r="K13" s="14">
         <f>A13*Assumptions!$B$17+B13*Assumptions!$B$18+Assumptions!$B$19</f>
-        <v/>
+        <v>300000</v>
       </c>
       <c r="L13" s="14">
         <f>K13*Assumptions!$B$20</f>
-        <v/>
+        <v>90000</v>
       </c>
       <c r="M13" s="14">
         <f>K13-L13-Assumptions!$B$21</f>
-        <v/>
+        <v>210000</v>
       </c>
       <c r="N13" s="13">
         <f>M13/J13</f>
-        <v/>
+        <v>26.98185586</v>
       </c>
       <c r="O13" s="14">
         <f>'CF_Calc'!U13</f>
-        <v/>
+        <v>-187879.2148</v>
       </c>
       <c r="P13" s="15">
         <f>'CF_Calc'!V13</f>
-        <v/>
+        <v>-0.1859918097</v>
       </c>
     </row>
     <row r="15">
@@ -3894,87 +3894,87 @@
       </c>
       <c r="B5">
         <f>'Sizing Comparison'!M5</f>
-        <v/>
+        <v>43400</v>
       </c>
       <c r="C5">
         <f>'Sizing Comparison'!J5</f>
-        <v/>
+        <v>3976.776</v>
       </c>
       <c r="D5">
         <f>'Sizing Comparison'!K5</f>
-        <v/>
+        <v>62000</v>
       </c>
       <c r="E5">
         <f>-B5</f>
-        <v/>
+        <v>-43400</v>
       </c>
       <c r="F5">
         <f>C5*(1+Assumptions!$B$7)^0*(1-Assumptions!$B$14*0)-D5*Assumptions!$B$38*(1+Assumptions!$B$39)^0</f>
-        <v/>
+        <v>3046.776</v>
       </c>
       <c r="G5">
         <f>C5*(1+Assumptions!$B$7)^1*(1-Assumptions!$B$14*1)-D5*Assumptions!$B$38*(1+Assumptions!$B$39)^1</f>
-        <v/>
+        <v>3025.690515</v>
       </c>
       <c r="H5">
         <f>C5*(1+Assumptions!$B$7)^2*(1-Assumptions!$B$14*2)-D5*Assumptions!$B$38*(1+Assumptions!$B$39)^2</f>
-        <v/>
+        <v>3001.623271</v>
       </c>
       <c r="I5">
         <f>C5*(1+Assumptions!$B$7)^3*(1-Assumptions!$B$14*3)-D5*Assumptions!$B$38*(1+Assumptions!$B$39)^3</f>
-        <v/>
+        <v>2974.437893</v>
       </c>
       <c r="J5">
         <f>C5*(1+Assumptions!$B$7)^4*(1-Assumptions!$B$14*4)-D5*Assumptions!$B$38*(1+Assumptions!$B$39)^4</f>
-        <v/>
+        <v>2943.993042</v>
       </c>
       <c r="K5">
         <f>C5*(1+Assumptions!$B$7)^5*(1-Assumptions!$B$14*5)-D5*Assumptions!$B$38*(1+Assumptions!$B$39)^5</f>
-        <v/>
+        <v>2910.142252</v>
       </c>
       <c r="L5">
         <f>C5*(1+Assumptions!$B$7)^6*(1-Assumptions!$B$14*6)-D5*Assumptions!$B$38*(1+Assumptions!$B$39)^6</f>
-        <v/>
+        <v>2872.73376</v>
       </c>
       <c r="M5">
         <f>C5*(1+Assumptions!$B$7)^7*(1-Assumptions!$B$14*7)-D5*Assumptions!$B$38*(1+Assumptions!$B$39)^7</f>
-        <v/>
+        <v>2831.610335</v>
       </c>
       <c r="N5">
         <f>C5*(1+Assumptions!$B$7)^8*(1-Assumptions!$B$14*8)-D5*Assumptions!$B$38*(1+Assumptions!$B$39)^8</f>
-        <v/>
+        <v>2786.609097</v>
       </c>
       <c r="O5">
         <f>C5*(1+Assumptions!$B$7)^9*(1-Assumptions!$B$14*9)-D5*Assumptions!$B$38*(1+Assumptions!$B$39)^9</f>
-        <v/>
+        <v>2737.561333</v>
       </c>
       <c r="P5">
         <f>C5*(1+Assumptions!$B$7)^10*(1-Assumptions!$B$14*10)-D5*Assumptions!$B$38*(1+Assumptions!$B$39)^10</f>
-        <v/>
+        <v>2684.292309</v>
       </c>
       <c r="Q5">
         <f>C5*(1+Assumptions!$B$7)^11*(1-Assumptions!$B$14*11)-D5*Assumptions!$B$38*(1+Assumptions!$B$39)^11</f>
-        <v/>
+        <v>2626.621073</v>
       </c>
       <c r="R5">
         <f>C5*(1+Assumptions!$B$7)^12*(1-Assumptions!$B$14*12)-D5*Assumptions!$B$38*(1+Assumptions!$B$39)^12</f>
-        <v/>
+        <v>2564.36025</v>
       </c>
       <c r="S5">
         <f>C5*(1+Assumptions!$B$7)^13*(1-Assumptions!$B$14*13)-D5*Assumptions!$B$38*(1+Assumptions!$B$39)^13</f>
-        <v/>
+        <v>2497.31584</v>
       </c>
       <c r="T5">
         <f>C5*(1+Assumptions!$B$7)^14*(1-Assumptions!$B$14*14)-D5*Assumptions!$B$38*(1+Assumptions!$B$39)^14</f>
-        <v/>
+        <v>2425.286997</v>
       </c>
       <c r="U5">
         <f>NPV(Assumptions!$B$40,F5:T5)+E5</f>
-        <v/>
+        <v>-18958.1907</v>
       </c>
       <c r="V5">
         <f>IFERROR(IRR(E5:T5),"-")</f>
-        <v/>
+        <v>-0.004440704189</v>
       </c>
     </row>
     <row r="6">
@@ -3985,87 +3985,87 @@
       </c>
       <c r="B6">
         <f>'Sizing Comparison'!M6</f>
-        <v/>
+        <v>63000</v>
       </c>
       <c r="C6">
         <f>'Sizing Comparison'!J6</f>
-        <v/>
+        <v>5160.248</v>
       </c>
       <c r="D6">
         <f>'Sizing Comparison'!K6</f>
-        <v/>
+        <v>90000</v>
       </c>
       <c r="E6">
         <f>-B6</f>
-        <v/>
+        <v>-63000</v>
       </c>
       <c r="F6">
         <f>C6*(1+Assumptions!$B$7)^0*(1-Assumptions!$B$14*0)-D6*Assumptions!$B$38*(1+Assumptions!$B$39)^0</f>
-        <v/>
+        <v>3810.248</v>
       </c>
       <c r="G6">
         <f>C6*(1+Assumptions!$B$7)^1*(1-Assumptions!$B$14*1)-D6*Assumptions!$B$38*(1+Assumptions!$B$39)^1</f>
-        <v/>
+        <v>3780.022845</v>
       </c>
       <c r="H6">
         <f>C6*(1+Assumptions!$B$7)^2*(1-Assumptions!$B$14*2)-D6*Assumptions!$B$38*(1+Assumptions!$B$39)^2</f>
-        <v/>
+        <v>3745.871277</v>
       </c>
       <c r="I6">
         <f>C6*(1+Assumptions!$B$7)^3*(1-Assumptions!$B$14*3)-D6*Assumptions!$B$38*(1+Assumptions!$B$39)^3</f>
-        <v/>
+        <v>3707.615192</v>
       </c>
       <c r="J6">
         <f>C6*(1+Assumptions!$B$7)^4*(1-Assumptions!$B$14*4)-D6*Assumptions!$B$38*(1+Assumptions!$B$39)^4</f>
-        <v/>
+        <v>3665.070019</v>
       </c>
       <c r="K6">
         <f>C6*(1+Assumptions!$B$7)^5*(1-Assumptions!$B$14*5)-D6*Assumptions!$B$38*(1+Assumptions!$B$39)^5</f>
-        <v/>
+        <v>3618.044512</v>
       </c>
       <c r="L6">
         <f>C6*(1+Assumptions!$B$7)^6*(1-Assumptions!$B$14*6)-D6*Assumptions!$B$38*(1+Assumptions!$B$39)^6</f>
-        <v/>
+        <v>3566.34053</v>
       </c>
       <c r="M6">
         <f>C6*(1+Assumptions!$B$7)^7*(1-Assumptions!$B$14*7)-D6*Assumptions!$B$38*(1+Assumptions!$B$39)^7</f>
-        <v/>
+        <v>3509.752807</v>
       </c>
       <c r="N6">
         <f>C6*(1+Assumptions!$B$7)^8*(1-Assumptions!$B$14*8)-D6*Assumptions!$B$38*(1+Assumptions!$B$39)^8</f>
-        <v/>
+        <v>3448.068728</v>
       </c>
       <c r="O6">
         <f>C6*(1+Assumptions!$B$7)^9*(1-Assumptions!$B$14*9)-D6*Assumptions!$B$38*(1+Assumptions!$B$39)^9</f>
-        <v/>
+        <v>3381.068081</v>
       </c>
       <c r="P6">
         <f>C6*(1+Assumptions!$B$7)^10*(1-Assumptions!$B$14*10)-D6*Assumptions!$B$38*(1+Assumptions!$B$39)^10</f>
-        <v/>
+        <v>3308.522815</v>
       </c>
       <c r="Q6">
         <f>C6*(1+Assumptions!$B$7)^11*(1-Assumptions!$B$14*11)-D6*Assumptions!$B$38*(1+Assumptions!$B$39)^11</f>
-        <v/>
+        <v>3230.196784</v>
       </c>
       <c r="R6">
         <f>C6*(1+Assumptions!$B$7)^12*(1-Assumptions!$B$14*12)-D6*Assumptions!$B$38*(1+Assumptions!$B$39)^12</f>
-        <v/>
+        <v>3145.845483</v>
       </c>
       <c r="S6">
         <f>C6*(1+Assumptions!$B$7)^13*(1-Assumptions!$B$14*13)-D6*Assumptions!$B$38*(1+Assumptions!$B$39)^13</f>
-        <v/>
+        <v>3055.215781</v>
       </c>
       <c r="T6">
         <f>C6*(1+Assumptions!$B$7)^14*(1-Assumptions!$B$14*14)-D6*Assumptions!$B$38*(1+Assumptions!$B$39)^14</f>
-        <v/>
+        <v>2958.045637</v>
       </c>
       <c r="U6">
         <f>NPV(Assumptions!$B$40,F6:T6)+E6</f>
-        <v/>
+        <v>-32658.82052</v>
       </c>
       <c r="V6">
         <f>IFERROR(IRR(E6:T6),"-")</f>
-        <v/>
+        <v>-0.02416452145</v>
       </c>
     </row>
     <row r="7">
@@ -4076,87 +4076,87 @@
       </c>
       <c r="B7">
         <f>'Sizing Comparison'!M7</f>
-        <v/>
+        <v>80500</v>
       </c>
       <c r="C7">
         <f>'Sizing Comparison'!J7</f>
-        <v/>
+        <v>6168.008</v>
       </c>
       <c r="D7">
         <f>'Sizing Comparison'!K7</f>
-        <v/>
+        <v>115000</v>
       </c>
       <c r="E7">
         <f>-B7</f>
-        <v/>
+        <v>-80500</v>
       </c>
       <c r="F7">
         <f>C7*(1+Assumptions!$B$7)^0*(1-Assumptions!$B$14*0)-D7*Assumptions!$B$38*(1+Assumptions!$B$39)^0</f>
-        <v/>
+        <v>4443.008</v>
       </c>
       <c r="G7">
         <f>C7*(1+Assumptions!$B$7)^1*(1-Assumptions!$B$14*1)-D7*Assumptions!$B$38*(1+Assumptions!$B$39)^1</f>
-        <v/>
+        <v>4404.652995</v>
       </c>
       <c r="H7">
         <f>C7*(1+Assumptions!$B$7)^2*(1-Assumptions!$B$14*2)-D7*Assumptions!$B$38*(1+Assumptions!$B$39)^2</f>
-        <v/>
+        <v>4361.560235</v>
       </c>
       <c r="I7">
         <f>C7*(1+Assumptions!$B$7)^3*(1-Assumptions!$B$14*3)-D7*Assumptions!$B$38*(1+Assumptions!$B$39)^3</f>
-        <v/>
+        <v>4313.515941</v>
       </c>
       <c r="J7">
         <f>C7*(1+Assumptions!$B$7)^4*(1-Assumptions!$B$14*4)-D7*Assumptions!$B$38*(1+Assumptions!$B$39)^4</f>
-        <v/>
+        <v>4260.29859</v>
       </c>
       <c r="K7">
         <f>C7*(1+Assumptions!$B$7)^5*(1-Assumptions!$B$14*5)-D7*Assumptions!$B$38*(1+Assumptions!$B$39)^5</f>
-        <v/>
+        <v>4201.678659</v>
       </c>
       <c r="L7">
         <f>C7*(1+Assumptions!$B$7)^6*(1-Assumptions!$B$14*6)-D7*Assumptions!$B$38*(1+Assumptions!$B$39)^6</f>
-        <v/>
+        <v>4137.418366</v>
       </c>
       <c r="M7">
         <f>C7*(1+Assumptions!$B$7)^7*(1-Assumptions!$B$14*7)-D7*Assumptions!$B$38*(1+Assumptions!$B$39)^7</f>
-        <v/>
+        <v>4067.271395</v>
       </c>
       <c r="N7">
         <f>C7*(1+Assumptions!$B$7)^8*(1-Assumptions!$B$14*8)-D7*Assumptions!$B$38*(1+Assumptions!$B$39)^8</f>
-        <v/>
+        <v>3990.982623</v>
       </c>
       <c r="O7">
         <f>C7*(1+Assumptions!$B$7)^9*(1-Assumptions!$B$14*9)-D7*Assumptions!$B$38*(1+Assumptions!$B$39)^9</f>
-        <v/>
+        <v>3908.287831</v>
       </c>
       <c r="P7">
         <f>C7*(1+Assumptions!$B$7)^10*(1-Assumptions!$B$14*10)-D7*Assumptions!$B$38*(1+Assumptions!$B$39)^10</f>
-        <v/>
+        <v>3818.913407</v>
       </c>
       <c r="Q7">
         <f>C7*(1+Assumptions!$B$7)^11*(1-Assumptions!$B$14*11)-D7*Assumptions!$B$38*(1+Assumptions!$B$39)^11</f>
-        <v/>
+        <v>3722.576044</v>
       </c>
       <c r="R7">
         <f>C7*(1+Assumptions!$B$7)^12*(1-Assumptions!$B$14*12)-D7*Assumptions!$B$38*(1+Assumptions!$B$39)^12</f>
-        <v/>
+        <v>3618.982423</v>
       </c>
       <c r="S7">
         <f>C7*(1+Assumptions!$B$7)^13*(1-Assumptions!$B$14*13)-D7*Assumptions!$B$38*(1+Assumptions!$B$39)^13</f>
-        <v/>
+        <v>3507.828891</v>
       </c>
       <c r="T7">
         <f>C7*(1+Assumptions!$B$7)^14*(1-Assumptions!$B$14*14)-D7*Assumptions!$B$38*(1+Assumptions!$B$39)^14</f>
-        <v/>
+        <v>3388.801124</v>
       </c>
       <c r="U7">
         <f>NPV(Assumptions!$B$40,F7:T7)+E7</f>
-        <v/>
+        <v>-45301.89769</v>
       </c>
       <c r="V7">
         <f>IFERROR(IRR(E7:T7),"-")</f>
-        <v/>
+        <v>-0.035832867</v>
       </c>
     </row>
     <row r="8">
@@ -4167,87 +4167,87 @@
       </c>
       <c r="B8">
         <f>'Sizing Comparison'!M8</f>
-        <v/>
+        <v>87500</v>
       </c>
       <c r="C8">
         <f>'Sizing Comparison'!J8</f>
-        <v/>
+        <v>6168.008</v>
       </c>
       <c r="D8">
         <f>'Sizing Comparison'!K8</f>
-        <v/>
+        <v>125000</v>
       </c>
       <c r="E8">
         <f>-B8</f>
-        <v/>
+        <v>-87500</v>
       </c>
       <c r="F8">
         <f>C8*(1+Assumptions!$B$7)^0*(1-Assumptions!$B$14*0)-D8*Assumptions!$B$38*(1+Assumptions!$B$39)^0</f>
-        <v/>
+        <v>4293.008</v>
       </c>
       <c r="G8">
         <f>C8*(1+Assumptions!$B$7)^1*(1-Assumptions!$B$14*1)-D8*Assumptions!$B$38*(1+Assumptions!$B$39)^1</f>
-        <v/>
+        <v>4251.652995</v>
       </c>
       <c r="H8">
         <f>C8*(1+Assumptions!$B$7)^2*(1-Assumptions!$B$14*2)-D8*Assumptions!$B$38*(1+Assumptions!$B$39)^2</f>
-        <v/>
+        <v>4205.500235</v>
       </c>
       <c r="I8">
         <f>C8*(1+Assumptions!$B$7)^3*(1-Assumptions!$B$14*3)-D8*Assumptions!$B$38*(1+Assumptions!$B$39)^3</f>
-        <v/>
+        <v>4154.334741</v>
       </c>
       <c r="J8">
         <f>C8*(1+Assumptions!$B$7)^4*(1-Assumptions!$B$14*4)-D8*Assumptions!$B$38*(1+Assumptions!$B$39)^4</f>
-        <v/>
+        <v>4097.933766</v>
       </c>
       <c r="K8">
         <f>C8*(1+Assumptions!$B$7)^5*(1-Assumptions!$B$14*5)-D8*Assumptions!$B$38*(1+Assumptions!$B$39)^5</f>
-        <v/>
+        <v>4036.066539</v>
       </c>
       <c r="L8">
         <f>C8*(1+Assumptions!$B$7)^6*(1-Assumptions!$B$14*6)-D8*Assumptions!$B$38*(1+Assumptions!$B$39)^6</f>
-        <v/>
+        <v>3968.494003</v>
       </c>
       <c r="M8">
         <f>C8*(1+Assumptions!$B$7)^7*(1-Assumptions!$B$14*7)-D8*Assumptions!$B$38*(1+Assumptions!$B$39)^7</f>
-        <v/>
+        <v>3894.968545</v>
       </c>
       <c r="N8">
         <f>C8*(1+Assumptions!$B$7)^8*(1-Assumptions!$B$14*8)-D8*Assumptions!$B$38*(1+Assumptions!$B$39)^8</f>
-        <v/>
+        <v>3815.233716</v>
       </c>
       <c r="O8">
         <f>C8*(1+Assumptions!$B$7)^9*(1-Assumptions!$B$14*9)-D8*Assumptions!$B$38*(1+Assumptions!$B$39)^9</f>
-        <v/>
+        <v>3729.023946</v>
       </c>
       <c r="P8">
         <f>C8*(1+Assumptions!$B$7)^10*(1-Assumptions!$B$14*10)-D8*Assumptions!$B$38*(1+Assumptions!$B$39)^10</f>
-        <v/>
+        <v>3636.064244</v>
       </c>
       <c r="Q8">
         <f>C8*(1+Assumptions!$B$7)^11*(1-Assumptions!$B$14*11)-D8*Assumptions!$B$38*(1+Assumptions!$B$39)^11</f>
-        <v/>
+        <v>3536.069898</v>
       </c>
       <c r="R8">
         <f>C8*(1+Assumptions!$B$7)^12*(1-Assumptions!$B$14*12)-D8*Assumptions!$B$38*(1+Assumptions!$B$39)^12</f>
-        <v/>
+        <v>3428.746154</v>
       </c>
       <c r="S8">
         <f>C8*(1+Assumptions!$B$7)^13*(1-Assumptions!$B$14*13)-D8*Assumptions!$B$38*(1+Assumptions!$B$39)^13</f>
-        <v/>
+        <v>3313.787896</v>
       </c>
       <c r="T8">
         <f>C8*(1+Assumptions!$B$7)^14*(1-Assumptions!$B$14*14)-D8*Assumptions!$B$38*(1+Assumptions!$B$39)^14</f>
-        <v/>
+        <v>3190.87931</v>
       </c>
       <c r="U8">
         <f>NPV(Assumptions!$B$40,F8:T8)+E8</f>
-        <v/>
+        <v>-53741.21312</v>
       </c>
       <c r="V8">
         <f>IFERROR(IRR(E8:T8),"-")</f>
-        <v/>
+        <v>-0.05043723692</v>
       </c>
     </row>
     <row r="9">
@@ -4258,87 +4258,87 @@
       </c>
       <c r="B9">
         <f>'Sizing Comparison'!M9</f>
-        <v/>
+        <v>112000</v>
       </c>
       <c r="C9">
         <f>'Sizing Comparison'!J9</f>
-        <v/>
+        <v>6744.24</v>
       </c>
       <c r="D9">
         <f>'Sizing Comparison'!K9</f>
-        <v/>
+        <v>160000</v>
       </c>
       <c r="E9">
         <f>-B9</f>
-        <v/>
+        <v>-112000</v>
       </c>
       <c r="F9">
         <f>C9*(1+Assumptions!$B$7)^0*(1-Assumptions!$B$14*0)-D9*Assumptions!$B$38*(1+Assumptions!$B$39)^0</f>
-        <v/>
+        <v>4344.24</v>
       </c>
       <c r="G9">
         <f>C9*(1+Assumptions!$B$7)^1*(1-Assumptions!$B$14*1)-D9*Assumptions!$B$38*(1+Assumptions!$B$39)^1</f>
-        <v/>
+        <v>4292.02485</v>
       </c>
       <c r="H9">
         <f>C9*(1+Assumptions!$B$7)^2*(1-Assumptions!$B$14*2)-D9*Assumptions!$B$38*(1+Assumptions!$B$39)^2</f>
-        <v/>
+        <v>4234.423792</v>
       </c>
       <c r="I9">
         <f>C9*(1+Assumptions!$B$7)^3*(1-Assumptions!$B$14*3)-D9*Assumptions!$B$38*(1+Assumptions!$B$39)^3</f>
-        <v/>
+        <v>4171.198967</v>
       </c>
       <c r="J9">
         <f>C9*(1+Assumptions!$B$7)^4*(1-Assumptions!$B$14*4)-D9*Assumptions!$B$38*(1+Assumptions!$B$39)^4</f>
-        <v/>
+        <v>4102.103961</v>
       </c>
       <c r="K9">
         <f>C9*(1+Assumptions!$B$7)^5*(1-Assumptions!$B$14*5)-D9*Assumptions!$B$38*(1+Assumptions!$B$39)^5</f>
-        <v/>
+        <v>4026.883532</v>
       </c>
       <c r="L9">
         <f>C9*(1+Assumptions!$B$7)^6*(1-Assumptions!$B$14*6)-D9*Assumptions!$B$38*(1+Assumptions!$B$39)^6</f>
-        <v/>
+        <v>3945.273322</v>
       </c>
       <c r="M9">
         <f>C9*(1+Assumptions!$B$7)^7*(1-Assumptions!$B$14*7)-D9*Assumptions!$B$38*(1+Assumptions!$B$39)^7</f>
-        <v/>
+        <v>3856.999554</v>
       </c>
       <c r="N9">
         <f>C9*(1+Assumptions!$B$7)^8*(1-Assumptions!$B$14*8)-D9*Assumptions!$B$38*(1+Assumptions!$B$39)^8</f>
-        <v/>
+        <v>3761.778732</v>
       </c>
       <c r="O9">
         <f>C9*(1+Assumptions!$B$7)^9*(1-Assumptions!$B$14*9)-D9*Assumptions!$B$38*(1+Assumptions!$B$39)^9</f>
-        <v/>
+        <v>3659.317323</v>
       </c>
       <c r="P9">
         <f>C9*(1+Assumptions!$B$7)^10*(1-Assumptions!$B$14*10)-D9*Assumptions!$B$38*(1+Assumptions!$B$39)^10</f>
-        <v/>
+        <v>3549.311432</v>
       </c>
       <c r="Q9">
         <f>C9*(1+Assumptions!$B$7)^11*(1-Assumptions!$B$14*11)-D9*Assumptions!$B$38*(1+Assumptions!$B$39)^11</f>
-        <v/>
+        <v>3431.446468</v>
       </c>
       <c r="R9">
         <f>C9*(1+Assumptions!$B$7)^12*(1-Assumptions!$B$14*12)-D9*Assumptions!$B$38*(1+Assumptions!$B$39)^12</f>
-        <v/>
+        <v>3305.396796</v>
       </c>
       <c r="S9">
         <f>C9*(1+Assumptions!$B$7)^13*(1-Assumptions!$B$14*13)-D9*Assumptions!$B$38*(1+Assumptions!$B$39)^13</f>
-        <v/>
+        <v>3170.825384</v>
       </c>
       <c r="T9">
         <f>C9*(1+Assumptions!$B$7)^14*(1-Assumptions!$B$14*14)-D9*Assumptions!$B$38*(1+Assumptions!$B$39)^14</f>
-        <v/>
+        <v>3027.383434</v>
       </c>
       <c r="U9">
         <f>NPV(Assumptions!$B$40,F9:T9)+E9</f>
-        <v/>
+        <v>-78444.1706</v>
       </c>
       <c r="V9">
         <f>IFERROR(IRR(E9:T9),"-")</f>
-        <v/>
+        <v>-0.07851302868</v>
       </c>
     </row>
     <row r="10">
@@ -4349,87 +4349,87 @@
       </c>
       <c r="B10">
         <f>'Sizing Comparison'!M10</f>
-        <v/>
+        <v>147000</v>
       </c>
       <c r="C10">
         <f>'Sizing Comparison'!J10</f>
-        <v/>
+        <v>7385.072</v>
       </c>
       <c r="D10">
         <f>'Sizing Comparison'!K10</f>
-        <v/>
+        <v>210000</v>
       </c>
       <c r="E10">
         <f>-B10</f>
-        <v/>
+        <v>-147000</v>
       </c>
       <c r="F10">
         <f>C10*(1+Assumptions!$B$7)^0*(1-Assumptions!$B$14*0)-D10*Assumptions!$B$38*(1+Assumptions!$B$39)^0</f>
-        <v/>
+        <v>4235.072</v>
       </c>
       <c r="G10">
         <f>C10*(1+Assumptions!$B$7)^1*(1-Assumptions!$B$14*1)-D10*Assumptions!$B$38*(1+Assumptions!$B$39)^1</f>
-        <v/>
+        <v>4167.45633</v>
       </c>
       <c r="H10">
         <f>C10*(1+Assumptions!$B$7)^2*(1-Assumptions!$B$14*2)-D10*Assumptions!$B$38*(1+Assumptions!$B$39)^2</f>
-        <v/>
+        <v>4093.734206</v>
       </c>
       <c r="I10">
         <f>C10*(1+Assumptions!$B$7)^3*(1-Assumptions!$B$14*3)-D10*Assumptions!$B$38*(1+Assumptions!$B$39)^3</f>
-        <v/>
+        <v>4013.640992</v>
       </c>
       <c r="J10">
         <f>C10*(1+Assumptions!$B$7)^4*(1-Assumptions!$B$14*4)-D10*Assumptions!$B$38*(1+Assumptions!$B$39)^4</f>
-        <v/>
+        <v>3926.902601</v>
       </c>
       <c r="K10">
         <f>C10*(1+Assumptions!$B$7)^5*(1-Assumptions!$B$14*5)-D10*Assumptions!$B$38*(1+Assumptions!$B$39)^5</f>
-        <v/>
+        <v>3833.235194</v>
       </c>
       <c r="L10">
         <f>C10*(1+Assumptions!$B$7)^6*(1-Assumptions!$B$14*6)-D10*Assumptions!$B$38*(1+Assumptions!$B$39)^6</f>
-        <v/>
+        <v>3732.344862</v>
       </c>
       <c r="M10">
         <f>C10*(1+Assumptions!$B$7)^7*(1-Assumptions!$B$14*7)-D10*Assumptions!$B$38*(1+Assumptions!$B$39)^7</f>
-        <v/>
+        <v>3623.927295</v>
       </c>
       <c r="N10">
         <f>C10*(1+Assumptions!$B$7)^8*(1-Assumptions!$B$14*8)-D10*Assumptions!$B$38*(1+Assumptions!$B$39)^8</f>
-        <v/>
+        <v>3507.667448</v>
       </c>
       <c r="O10">
         <f>C10*(1+Assumptions!$B$7)^9*(1-Assumptions!$B$14*9)-D10*Assumptions!$B$38*(1+Assumptions!$B$39)^9</f>
-        <v/>
+        <v>3383.239196</v>
       </c>
       <c r="P10">
         <f>C10*(1+Assumptions!$B$7)^10*(1-Assumptions!$B$14*10)-D10*Assumptions!$B$38*(1+Assumptions!$B$39)^10</f>
-        <v/>
+        <v>3250.304971</v>
       </c>
       <c r="Q10">
         <f>C10*(1+Assumptions!$B$7)^11*(1-Assumptions!$B$14*11)-D10*Assumptions!$B$38*(1+Assumptions!$B$39)^11</f>
-        <v/>
+        <v>3108.515396</v>
       </c>
       <c r="R10">
         <f>C10*(1+Assumptions!$B$7)^12*(1-Assumptions!$B$14*12)-D10*Assumptions!$B$38*(1+Assumptions!$B$39)^12</f>
-        <v/>
+        <v>2957.508906</v>
       </c>
       <c r="S10">
         <f>C10*(1+Assumptions!$B$7)^13*(1-Assumptions!$B$14*13)-D10*Assumptions!$B$38*(1+Assumptions!$B$39)^13</f>
-        <v/>
+        <v>2796.911354</v>
       </c>
       <c r="T10">
         <f>C10*(1+Assumptions!$B$7)^14*(1-Assumptions!$B$14*14)-D10*Assumptions!$B$38*(1+Assumptions!$B$39)^14</f>
-        <v/>
+        <v>2626.335608</v>
       </c>
       <c r="U10">
         <f>NPV(Assumptions!$B$40,F10:T10)+E10</f>
-        <v/>
+        <v>-115264.1005</v>
       </c>
       <c r="V10">
         <f>IFERROR(IRR(E10:T10),"-")</f>
-        <v/>
+        <v>-0.1128356093</v>
       </c>
     </row>
     <row r="11">
@@ -4440,87 +4440,87 @@
       </c>
       <c r="B11">
         <f>'Sizing Comparison'!M11</f>
-        <v/>
+        <v>182000</v>
       </c>
       <c r="C11">
         <f>'Sizing Comparison'!J11</f>
-        <v/>
+        <v>7783.008</v>
       </c>
       <c r="D11">
         <f>'Sizing Comparison'!K11</f>
-        <v/>
+        <v>260000</v>
       </c>
       <c r="E11">
         <f>-B11</f>
-        <v/>
+        <v>-182000</v>
       </c>
       <c r="F11">
         <f>C11*(1+Assumptions!$B$7)^0*(1-Assumptions!$B$14*0)-D11*Assumptions!$B$38*(1+Assumptions!$B$39)^0</f>
-        <v/>
+        <v>3883.008</v>
       </c>
       <c r="G11">
         <f>C11*(1+Assumptions!$B$7)^1*(1-Assumptions!$B$14*1)-D11*Assumptions!$B$38*(1+Assumptions!$B$39)^1</f>
-        <v/>
+        <v>3800.14362</v>
       </c>
       <c r="H11">
         <f>C11*(1+Assumptions!$B$7)^2*(1-Assumptions!$B$14*2)-D11*Assumptions!$B$38*(1+Assumptions!$B$39)^2</f>
-        <v/>
+        <v>3710.611641</v>
       </c>
       <c r="I11">
         <f>C11*(1+Assumptions!$B$7)^3*(1-Assumptions!$B$14*3)-D11*Assumptions!$B$38*(1+Assumptions!$B$39)^3</f>
-        <v/>
+        <v>3614.128523</v>
       </c>
       <c r="J11">
         <f>C11*(1+Assumptions!$B$7)^4*(1-Assumptions!$B$14*4)-D11*Assumptions!$B$38*(1+Assumptions!$B$39)^4</f>
-        <v/>
+        <v>3510.400678</v>
       </c>
       <c r="K11">
         <f>C11*(1+Assumptions!$B$7)^5*(1-Assumptions!$B$14*5)-D11*Assumptions!$B$38*(1+Assumptions!$B$39)^5</f>
-        <v/>
+        <v>3399.124143</v>
       </c>
       <c r="L11">
         <f>C11*(1+Assumptions!$B$7)^6*(1-Assumptions!$B$14*6)-D11*Assumptions!$B$38*(1+Assumptions!$B$39)^6</f>
-        <v/>
+        <v>3279.984244</v>
       </c>
       <c r="M11">
         <f>C11*(1+Assumptions!$B$7)^7*(1-Assumptions!$B$14*7)-D11*Assumptions!$B$38*(1+Assumptions!$B$39)^7</f>
-        <v/>
+        <v>3152.655249</v>
       </c>
       <c r="N11">
         <f>C11*(1+Assumptions!$B$7)^8*(1-Assumptions!$B$14*8)-D11*Assumptions!$B$38*(1+Assumptions!$B$39)^8</f>
-        <v/>
+        <v>3016.800013</v>
       </c>
       <c r="O11">
         <f>C11*(1+Assumptions!$B$7)^9*(1-Assumptions!$B$14*9)-D11*Assumptions!$B$38*(1+Assumptions!$B$39)^9</f>
-        <v/>
+        <v>2872.069609</v>
       </c>
       <c r="P11">
         <f>C11*(1+Assumptions!$B$7)^10*(1-Assumptions!$B$14*10)-D11*Assumptions!$B$38*(1+Assumptions!$B$39)^10</f>
-        <v/>
+        <v>2718.102948</v>
       </c>
       <c r="Q11">
         <f>C11*(1+Assumptions!$B$7)^11*(1-Assumptions!$B$14*11)-D11*Assumptions!$B$38*(1+Assumptions!$B$39)^11</f>
-        <v/>
+        <v>2554.526389</v>
       </c>
       <c r="R11">
         <f>C11*(1+Assumptions!$B$7)^12*(1-Assumptions!$B$14*12)-D11*Assumptions!$B$38*(1+Assumptions!$B$39)^12</f>
-        <v/>
+        <v>2380.953336</v>
       </c>
       <c r="S11">
         <f>C11*(1+Assumptions!$B$7)^13*(1-Assumptions!$B$14*13)-D11*Assumptions!$B$38*(1+Assumptions!$B$39)^13</f>
-        <v/>
+        <v>2196.983822</v>
       </c>
       <c r="T11">
         <f>C11*(1+Assumptions!$B$7)^14*(1-Assumptions!$B$14*14)-D11*Assumptions!$B$38*(1+Assumptions!$B$39)^14</f>
-        <v/>
+        <v>2002.204083</v>
       </c>
       <c r="U11">
         <f>NPV(Assumptions!$B$40,F11:T11)+E11</f>
-        <v/>
+        <v>-154121.9531</v>
       </c>
       <c r="V11">
         <f>IFERROR(IRR(E11:T11),"-")</f>
-        <v/>
+        <v>-0.1475420424</v>
       </c>
     </row>
     <row r="12">
@@ -4531,87 +4531,87 @@
       </c>
       <c r="B12">
         <f>'Sizing Comparison'!M12</f>
-        <v/>
+        <v>161000</v>
       </c>
       <c r="C12">
         <f>'Sizing Comparison'!J12</f>
-        <v/>
+        <v>7385.072</v>
       </c>
       <c r="D12">
         <f>'Sizing Comparison'!K12</f>
-        <v/>
+        <v>230000</v>
       </c>
       <c r="E12">
         <f>-B12</f>
-        <v/>
+        <v>-161000</v>
       </c>
       <c r="F12">
         <f>C12*(1+Assumptions!$B$7)^0*(1-Assumptions!$B$14*0)-D12*Assumptions!$B$38*(1+Assumptions!$B$39)^0</f>
-        <v/>
+        <v>3935.072</v>
       </c>
       <c r="G12">
         <f>C12*(1+Assumptions!$B$7)^1*(1-Assumptions!$B$14*1)-D12*Assumptions!$B$38*(1+Assumptions!$B$39)^1</f>
-        <v/>
+        <v>3861.45633</v>
       </c>
       <c r="H12">
         <f>C12*(1+Assumptions!$B$7)^2*(1-Assumptions!$B$14*2)-D12*Assumptions!$B$38*(1+Assumptions!$B$39)^2</f>
-        <v/>
+        <v>3781.614206</v>
       </c>
       <c r="I12">
         <f>C12*(1+Assumptions!$B$7)^3*(1-Assumptions!$B$14*3)-D12*Assumptions!$B$38*(1+Assumptions!$B$39)^3</f>
-        <v/>
+        <v>3695.278592</v>
       </c>
       <c r="J12">
         <f>C12*(1+Assumptions!$B$7)^4*(1-Assumptions!$B$14*4)-D12*Assumptions!$B$38*(1+Assumptions!$B$39)^4</f>
-        <v/>
+        <v>3602.172953</v>
       </c>
       <c r="K12">
         <f>C12*(1+Assumptions!$B$7)^5*(1-Assumptions!$B$14*5)-D12*Assumptions!$B$38*(1+Assumptions!$B$39)^5</f>
-        <v/>
+        <v>3502.010953</v>
       </c>
       <c r="L12">
         <f>C12*(1+Assumptions!$B$7)^6*(1-Assumptions!$B$14*6)-D12*Assumptions!$B$38*(1+Assumptions!$B$39)^6</f>
-        <v/>
+        <v>3394.496136</v>
       </c>
       <c r="M12">
         <f>C12*(1+Assumptions!$B$7)^7*(1-Assumptions!$B$14*7)-D12*Assumptions!$B$38*(1+Assumptions!$B$39)^7</f>
-        <v/>
+        <v>3279.321594</v>
       </c>
       <c r="N12">
         <f>C12*(1+Assumptions!$B$7)^8*(1-Assumptions!$B$14*8)-D12*Assumptions!$B$38*(1+Assumptions!$B$39)^8</f>
-        <v/>
+        <v>3156.169634</v>
       </c>
       <c r="O12">
         <f>C12*(1+Assumptions!$B$7)^9*(1-Assumptions!$B$14*9)-D12*Assumptions!$B$38*(1+Assumptions!$B$39)^9</f>
-        <v/>
+        <v>3024.711425</v>
       </c>
       <c r="P12">
         <f>C12*(1+Assumptions!$B$7)^10*(1-Assumptions!$B$14*10)-D12*Assumptions!$B$38*(1+Assumptions!$B$39)^10</f>
-        <v/>
+        <v>2884.606645</v>
       </c>
       <c r="Q12">
         <f>C12*(1+Assumptions!$B$7)^11*(1-Assumptions!$B$14*11)-D12*Assumptions!$B$38*(1+Assumptions!$B$39)^11</f>
-        <v/>
+        <v>2735.503104</v>
       </c>
       <c r="R12">
         <f>C12*(1+Assumptions!$B$7)^12*(1-Assumptions!$B$14*12)-D12*Assumptions!$B$38*(1+Assumptions!$B$39)^12</f>
-        <v/>
+        <v>2577.036368</v>
       </c>
       <c r="S12">
         <f>C12*(1+Assumptions!$B$7)^13*(1-Assumptions!$B$14*13)-D12*Assumptions!$B$38*(1+Assumptions!$B$39)^13</f>
-        <v/>
+        <v>2408.829365</v>
       </c>
       <c r="T12">
         <f>C12*(1+Assumptions!$B$7)^14*(1-Assumptions!$B$14*14)-D12*Assumptions!$B$38*(1+Assumptions!$B$39)^14</f>
-        <v/>
+        <v>2230.491979</v>
       </c>
       <c r="U12">
         <f>NPV(Assumptions!$B$40,F12:T12)+E12</f>
-        <v/>
+        <v>-132142.7313</v>
       </c>
       <c r="V12">
         <f>IFERROR(IRR(E12:T12),"-")</f>
-        <v/>
+        <v>-0.131715269</v>
       </c>
     </row>
     <row r="13">
@@ -4622,87 +4622,87 @@
       </c>
       <c r="B13">
         <f>'Sizing Comparison'!M13</f>
-        <v/>
+        <v>210000</v>
       </c>
       <c r="C13">
         <f>'Sizing Comparison'!J13</f>
-        <v/>
+        <v>7783.008</v>
       </c>
       <c r="D13">
         <f>'Sizing Comparison'!K13</f>
-        <v/>
+        <v>300000</v>
       </c>
       <c r="E13">
         <f>-B13</f>
-        <v/>
+        <v>-210000</v>
       </c>
       <c r="F13">
         <f>C13*(1+Assumptions!$B$7)^0*(1-Assumptions!$B$14*0)-D13*Assumptions!$B$38*(1+Assumptions!$B$39)^0</f>
-        <v/>
+        <v>3283.008</v>
       </c>
       <c r="G13">
         <f>C13*(1+Assumptions!$B$7)^1*(1-Assumptions!$B$14*1)-D13*Assumptions!$B$38*(1+Assumptions!$B$39)^1</f>
-        <v/>
+        <v>3188.14362</v>
       </c>
       <c r="H13">
         <f>C13*(1+Assumptions!$B$7)^2*(1-Assumptions!$B$14*2)-D13*Assumptions!$B$38*(1+Assumptions!$B$39)^2</f>
-        <v/>
+        <v>3086.371641</v>
       </c>
       <c r="I13">
         <f>C13*(1+Assumptions!$B$7)^3*(1-Assumptions!$B$14*3)-D13*Assumptions!$B$38*(1+Assumptions!$B$39)^3</f>
-        <v/>
+        <v>2977.403723</v>
       </c>
       <c r="J13">
         <f>C13*(1+Assumptions!$B$7)^4*(1-Assumptions!$B$14*4)-D13*Assumptions!$B$38*(1+Assumptions!$B$39)^4</f>
-        <v/>
+        <v>2860.941382</v>
       </c>
       <c r="K13">
         <f>C13*(1+Assumptions!$B$7)^5*(1-Assumptions!$B$14*5)-D13*Assumptions!$B$38*(1+Assumptions!$B$39)^5</f>
-        <v/>
+        <v>2736.675661</v>
       </c>
       <c r="L13">
         <f>C13*(1+Assumptions!$B$7)^6*(1-Assumptions!$B$14*6)-D13*Assumptions!$B$38*(1+Assumptions!$B$39)^6</f>
-        <v/>
+        <v>2604.286792</v>
       </c>
       <c r="M13">
         <f>C13*(1+Assumptions!$B$7)^7*(1-Assumptions!$B$14*7)-D13*Assumptions!$B$38*(1+Assumptions!$B$39)^7</f>
-        <v/>
+        <v>2463.443848</v>
       </c>
       <c r="N13">
         <f>C13*(1+Assumptions!$B$7)^8*(1-Assumptions!$B$14*8)-D13*Assumptions!$B$38*(1+Assumptions!$B$39)^8</f>
-        <v/>
+        <v>2313.804384</v>
       </c>
       <c r="O13">
         <f>C13*(1+Assumptions!$B$7)^9*(1-Assumptions!$B$14*9)-D13*Assumptions!$B$38*(1+Assumptions!$B$39)^9</f>
-        <v/>
+        <v>2155.014068</v>
       </c>
       <c r="P13">
         <f>C13*(1+Assumptions!$B$7)^10*(1-Assumptions!$B$14*10)-D13*Assumptions!$B$38*(1+Assumptions!$B$39)^10</f>
-        <v/>
+        <v>1986.706296</v>
       </c>
       <c r="Q13">
         <f>C13*(1+Assumptions!$B$7)^11*(1-Assumptions!$B$14*11)-D13*Assumptions!$B$38*(1+Assumptions!$B$39)^11</f>
-        <v/>
+        <v>1808.501804</v>
       </c>
       <c r="R13">
         <f>C13*(1+Assumptions!$B$7)^12*(1-Assumptions!$B$14*12)-D13*Assumptions!$B$38*(1+Assumptions!$B$39)^12</f>
-        <v/>
+        <v>1620.008259</v>
       </c>
       <c r="S13">
         <f>C13*(1+Assumptions!$B$7)^13*(1-Assumptions!$B$14*13)-D13*Assumptions!$B$38*(1+Assumptions!$B$39)^13</f>
-        <v/>
+        <v>1420.819844</v>
       </c>
       <c r="T13">
         <f>C13*(1+Assumptions!$B$7)^14*(1-Assumptions!$B$14*14)-D13*Assumptions!$B$38*(1+Assumptions!$B$39)^14</f>
-        <v/>
+        <v>1210.516825</v>
       </c>
       <c r="U13">
         <f>NPV(Assumptions!$B$40,F13:T13)+E13</f>
-        <v/>
+        <v>-187879.2148</v>
       </c>
       <c r="V13">
         <f>IFERROR(IRR(E13:T13),"-")</f>
-        <v/>
+        <v>-0.1859918097</v>
       </c>
     </row>
   </sheetData>
@@ -4800,19 +4800,19 @@
       </c>
       <c r="D6" s="26">
         <f>Assumptions!$B$32*Assumptions!$B$33*C6</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E6" s="26">
         <f>MIN(D6,B6)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F6" s="26">
         <f>D6-E6</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G6" s="14">
         <f>E6*Assumptions!$B$4+F6*Assumptions!$B$35</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -4829,19 +4829,19 @@
       </c>
       <c r="D7" s="26">
         <f>Assumptions!$B$32*Assumptions!$B$33*C7</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E7" s="26">
         <f>MIN(D7,B7)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F7" s="26">
         <f>D7-E7</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G7" s="14">
         <f>E7*Assumptions!$B$4+F7*Assumptions!$B$35</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -4858,19 +4858,19 @@
       </c>
       <c r="D8" s="26">
         <f>Assumptions!$B$32*Assumptions!$B$33*C8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E8" s="26">
         <f>MIN(D8,B8)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F8" s="26">
         <f>D8-E8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G8" s="14">
         <f>E8*Assumptions!$B$4+F8*Assumptions!$B$35</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -4887,19 +4887,19 @@
       </c>
       <c r="D9" s="26">
         <f>Assumptions!$B$32*Assumptions!$B$33*C9</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E9" s="26">
         <f>MIN(D9,B9)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F9" s="26">
         <f>D9-E9</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G9" s="14">
         <f>E9*Assumptions!$B$4+F9*Assumptions!$B$35</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -4916,19 +4916,19 @@
       </c>
       <c r="D10" s="26">
         <f>Assumptions!$B$32*Assumptions!$B$33*C10</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E10" s="26">
         <f>MIN(D10,B10)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F10" s="26">
         <f>D10-E10</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G10" s="14">
         <f>E10*Assumptions!$B$4+F10*Assumptions!$B$35</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -4945,19 +4945,19 @@
       </c>
       <c r="D11" s="26">
         <f>Assumptions!$B$32*Assumptions!$B$33*C11</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E11" s="26">
         <f>MIN(D11,B11)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F11" s="26">
         <f>D11-E11</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G11" s="14">
         <f>E11*Assumptions!$B$4+F11*Assumptions!$B$35</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -4974,19 +4974,19 @@
       </c>
       <c r="D12" s="26">
         <f>Assumptions!$B$32*Assumptions!$B$33*C12</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E12" s="26">
         <f>MIN(D12,B12)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F12" s="26">
         <f>D12-E12</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G12" s="14">
         <f>E12*Assumptions!$B$4+F12*Assumptions!$B$35</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -5003,19 +5003,19 @@
       </c>
       <c r="D13" s="26">
         <f>Assumptions!$B$32*Assumptions!$B$33*C13</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E13" s="26">
         <f>MIN(D13,B13)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F13" s="26">
         <f>D13-E13</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G13" s="14">
         <f>E13*Assumptions!$B$4+F13*Assumptions!$B$35</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -5032,19 +5032,19 @@
       </c>
       <c r="D14" s="26">
         <f>Assumptions!$B$32*Assumptions!$B$33*C14</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E14" s="26">
         <f>MIN(D14,B14)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F14" s="26">
         <f>D14-E14</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G14" s="14">
         <f>E14*Assumptions!$B$4+F14*Assumptions!$B$35</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -5061,19 +5061,19 @@
       </c>
       <c r="D15" s="26">
         <f>Assumptions!$B$32*Assumptions!$B$33*C15</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E15" s="26">
         <f>MIN(D15,B15)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F15" s="26">
         <f>D15-E15</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G15" s="14">
         <f>E15*Assumptions!$B$4+F15*Assumptions!$B$35</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -5090,19 +5090,19 @@
       </c>
       <c r="D16" s="26">
         <f>Assumptions!$B$32*Assumptions!$B$33*C16</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E16" s="26">
         <f>MIN(D16,B16)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F16" s="26">
         <f>D16-E16</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G16" s="14">
         <f>E16*Assumptions!$B$4+F16*Assumptions!$B$35</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -5119,19 +5119,19 @@
       </c>
       <c r="D17" s="26">
         <f>Assumptions!$B$32*Assumptions!$B$33*C17</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E17" s="26">
         <f>MIN(D17,B17)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F17" s="26">
         <f>D17-E17</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G17" s="14">
         <f>E17*Assumptions!$B$4+F17*Assumptions!$B$35</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -5148,15 +5148,15 @@
       </c>
       <c r="E18" s="28">
         <f>SUM(E6:E17)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F18" s="28">
         <f>SUM(F6:F17)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G18" s="29">
         <f>SUM(G6:G17)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -5167,7 +5167,7 @@
       </c>
       <c r="B20" s="31">
         <f>Assumptions!$B$32*Assumptions!$B$34</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -5178,7 +5178,7 @@
       </c>
       <c r="B21" s="31">
         <f>B20*(1-Assumptions!$B$20)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -5189,7 +5189,7 @@
       </c>
       <c r="B22" s="31">
         <f>G18</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -5198,9 +5198,9 @@
           <t>PV simple payback (yr)</t>
         </is>
       </c>
-      <c r="B23" s="32">
+      <c t="str" r="B23" s="32">
         <f>IFERROR(B21/B22,"-")</f>
-        <v/>
+        <v>-</v>
       </c>
     </row>
     <row r="24">
@@ -5211,7 +5211,7 @@
       </c>
       <c r="B24" s="33">
         <f>IFERROR(E18/D18,0)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5269,7 +5269,7 @@
       </c>
       <c r="B5" s="14">
         <f>'Sizing Comparison'!E7</f>
-        <v/>
+        <v>6168.008</v>
       </c>
     </row>
     <row r="6">
@@ -5280,7 +5280,7 @@
       </c>
       <c r="B6" s="14">
         <f>'Sizing Comparison'!F7</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -5291,7 +5291,7 @@
       </c>
       <c r="B7" s="14">
         <f>'Sizing Comparison'!G7</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -5302,7 +5302,7 @@
       </c>
       <c r="B8" s="14">
         <f>'Sizing Comparison'!H7</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -5313,7 +5313,7 @@
       </c>
       <c r="B9" s="14">
         <f>'Sizing Comparison'!I7</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -5324,7 +5324,7 @@
       </c>
       <c r="B10" s="14">
         <f>'Solar + Storage'!B22</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -5335,7 +5335,7 @@
       </c>
       <c r="B11" s="34">
         <f>SUM(B5:B10)</f>
-        <v/>
+        <v>6168.008</v>
       </c>
     </row>
     <row r="13">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="B13" s="31">
         <f>'Sizing Comparison'!M7</f>
-        <v/>
+        <v>80500</v>
       </c>
     </row>
     <row r="14">
@@ -5357,7 +5357,7 @@
       </c>
       <c r="B14" s="31">
         <f>'Solar + Storage'!B21</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -5368,7 +5368,7 @@
       </c>
       <c r="B15" s="31">
         <f>B13+B14</f>
-        <v/>
+        <v>80500</v>
       </c>
     </row>
     <row r="17">
@@ -5379,7 +5379,7 @@
       </c>
       <c r="B17" s="36">
         <f>IFERROR(B15/B11,"-")</f>
-        <v/>
+        <v>13.05121524</v>
       </c>
     </row>
   </sheetData>
@@ -5445,7 +5445,7 @@
       </c>
       <c r="B6" s="33">
         <f>B5/B4</f>
-        <v/>
+        <v>0.2236727589</v>
       </c>
     </row>
     <row r="9">
@@ -5494,15 +5494,15 @@
       </c>
       <c r="D10" s="14">
         <f>C10*Assumptions!$B$5</f>
-        <v/>
+        <v>2090.456</v>
       </c>
       <c r="E10" s="14">
         <f>B10*Assumptions!$B$4</f>
-        <v/>
+        <v>3989.9602</v>
       </c>
       <c r="F10" s="14">
         <f>D10+E10</f>
-        <v/>
+        <v>6080.4162</v>
       </c>
     </row>
     <row r="11">
@@ -5519,15 +5519,15 @@
       </c>
       <c r="D11" s="14">
         <f>C11*Assumptions!$B$5</f>
-        <v/>
+        <v>2341.104</v>
       </c>
       <c r="E11" s="14">
         <f>B11*Assumptions!$B$4</f>
-        <v/>
+        <v>3817.2889</v>
       </c>
       <c r="F11" s="14">
         <f>D11+E11</f>
-        <v/>
+        <v>6158.3929</v>
       </c>
     </row>
     <row r="12">
@@ -5544,15 +5544,15 @@
       </c>
       <c r="D12" s="14">
         <f>C12*Assumptions!$B$5</f>
-        <v/>
+        <v>2904.416</v>
       </c>
       <c r="E12" s="14">
         <f>B12*Assumptions!$B$4</f>
-        <v/>
+        <v>4774.3559</v>
       </c>
       <c r="F12" s="14">
         <f>D12+E12</f>
-        <v/>
+        <v>7678.7719</v>
       </c>
     </row>
     <row r="13">
@@ -5569,15 +5569,15 @@
       </c>
       <c r="D13" s="14">
         <f>C13*Assumptions!$B$5</f>
-        <v/>
+        <v>2098.208</v>
       </c>
       <c r="E13" s="14">
         <f>B13*Assumptions!$B$4</f>
-        <v/>
+        <v>3119.9497</v>
       </c>
       <c r="F13" s="14">
         <f>D13+E13</f>
-        <v/>
+        <v>5218.1577</v>
       </c>
     </row>
     <row r="14">
@@ -5594,15 +5594,15 @@
       </c>
       <c r="D14" s="14">
         <f>C14*Assumptions!$B$5</f>
-        <v/>
+        <v>762.28</v>
       </c>
       <c r="E14" s="14">
         <f>B14*Assumptions!$B$4</f>
-        <v/>
+        <v>692.5705</v>
       </c>
       <c r="F14" s="14">
         <f>D14+E14</f>
-        <v/>
+        <v>1454.8505</v>
       </c>
     </row>
     <row r="15">
@@ -5619,15 +5619,15 @@
       </c>
       <c r="D15" s="14">
         <f>C15*Assumptions!$B$5</f>
-        <v/>
+        <v>684.76</v>
       </c>
       <c r="E15" s="14">
         <f>B15*Assumptions!$B$4</f>
-        <v/>
+        <v>528.4385</v>
       </c>
       <c r="F15" s="14">
         <f>D15+E15</f>
-        <v/>
+        <v>1213.1985</v>
       </c>
     </row>
     <row r="16">
@@ -5644,15 +5644,15 @@
       </c>
       <c r="D16" s="14">
         <f>C16*Assumptions!$B$5</f>
-        <v/>
+        <v>550.392</v>
       </c>
       <c r="E16" s="14">
         <f>B16*Assumptions!$B$4</f>
-        <v/>
+        <v>478.6444</v>
       </c>
       <c r="F16" s="14">
         <f>D16+E16</f>
-        <v/>
+        <v>1029.0364</v>
       </c>
     </row>
     <row r="17">
@@ -5669,15 +5669,15 @@
       </c>
       <c r="D17" s="14">
         <f>C17*Assumptions!$B$5</f>
-        <v/>
+        <v>620.16</v>
       </c>
       <c r="E17" s="14">
         <f>B17*Assumptions!$B$4</f>
-        <v/>
+        <v>384.6012</v>
       </c>
       <c r="F17" s="14">
         <f>D17+E17</f>
-        <v/>
+        <v>1004.7612</v>
       </c>
     </row>
     <row r="18">
@@ -5694,15 +5694,15 @@
       </c>
       <c r="D18" s="14">
         <f>C18*Assumptions!$B$5</f>
-        <v/>
+        <v>436.696</v>
       </c>
       <c r="E18" s="14">
         <f>B18*Assumptions!$B$4</f>
-        <v/>
+        <v>324.6043</v>
       </c>
       <c r="F18" s="14">
         <f>D18+E18</f>
-        <v/>
+        <v>761.3003</v>
       </c>
     </row>
     <row r="19">
@@ -5719,15 +5719,15 @@
       </c>
       <c r="D19" s="14">
         <f>C19*Assumptions!$B$5</f>
-        <v/>
+        <v>475.456</v>
       </c>
       <c r="E19" s="14">
         <f>B19*Assumptions!$B$4</f>
-        <v/>
+        <v>289.0054</v>
       </c>
       <c r="F19" s="14">
         <f>D19+E19</f>
-        <v/>
+        <v>764.4614</v>
       </c>
     </row>
     <row r="20">
@@ -5744,15 +5744,15 @@
       </c>
       <c r="D20" s="14">
         <f>C20*Assumptions!$B$5</f>
-        <v/>
+        <v>2969.016</v>
       </c>
       <c r="E20" s="14">
         <f>B20*Assumptions!$B$4</f>
-        <v/>
+        <v>3843.5722</v>
       </c>
       <c r="F20" s="14">
         <f>D20+E20</f>
-        <v/>
+        <v>6812.5882</v>
       </c>
     </row>
     <row r="21">
@@ -5769,15 +5769,15 @@
       </c>
       <c r="D21" s="14">
         <f>C21*Assumptions!$B$5</f>
-        <v/>
+        <v>1832.056</v>
       </c>
       <c r="E21" s="14">
         <f>B21*Assumptions!$B$4</f>
-        <v/>
+        <v>2679.1222</v>
       </c>
       <c r="F21" s="14">
         <f>D21+E21</f>
-        <v/>
+        <v>4511.1782</v>
       </c>
     </row>
     <row r="22">
@@ -5788,7 +5788,7 @@
       </c>
       <c r="B22" s="27">
         <f>SUM(B10:B21)</f>
-        <v/>
+        <v>224726</v>
       </c>
       <c r="C22" s="12" t="n"/>
       <c r="D22" s="29">
@@ -5797,11 +5797,11 @@
       </c>
       <c r="E22" s="29">
         <f>SUM(E10:E21)</f>
-        <v/>
+        <v>24922.1134</v>
       </c>
       <c r="F22" s="29">
         <f>SUM(F10:F21)</f>
-        <v/>
+        <v>42687.1134</v>
       </c>
     </row>
   </sheetData>
@@ -5886,19 +5886,19 @@
       </c>
       <c r="D4" s="12">
         <f>B4-C4</f>
-        <v/>
+        <v>26.2</v>
       </c>
       <c r="E4" s="14">
         <f>B4*Assumptions!$B$5+35978*Assumptions!$B$4</f>
-        <v/>
+        <v>6080.4162</v>
       </c>
       <c r="F4" s="14">
         <f>C4*Assumptions!$B$5+35978*Assumptions!$B$4</f>
-        <v/>
+        <v>5403.4082</v>
       </c>
       <c r="G4" s="14">
         <f>E4-F4</f>
-        <v/>
+        <v>677.008</v>
       </c>
     </row>
     <row r="5">
@@ -5915,19 +5915,19 @@
       </c>
       <c r="D5" s="12">
         <f>B5-C5</f>
-        <v/>
+        <v>32.1</v>
       </c>
       <c r="E5" s="14">
         <f>B5*Assumptions!$B$5+34421*Assumptions!$B$4</f>
-        <v/>
+        <v>6158.3929</v>
       </c>
       <c r="F5" s="14">
         <f>C5*Assumptions!$B$5+34421*Assumptions!$B$4</f>
-        <v/>
+        <v>5328.9289</v>
       </c>
       <c r="G5" s="14">
         <f>E5-F5</f>
-        <v/>
+        <v>829.464</v>
       </c>
     </row>
     <row r="6">
@@ -5944,19 +5944,19 @@
       </c>
       <c r="D6" s="12">
         <f>B6-C6</f>
-        <v/>
+        <v>18.8</v>
       </c>
       <c r="E6" s="14">
         <f>B6*Assumptions!$B$5+43051*Assumptions!$B$4</f>
-        <v/>
+        <v>7678.7719</v>
       </c>
       <c r="F6" s="14">
         <f>C6*Assumptions!$B$5+43051*Assumptions!$B$4</f>
-        <v/>
+        <v>7192.9799</v>
       </c>
       <c r="G6" s="14">
         <f>E6-F6</f>
-        <v/>
+        <v>485.792</v>
       </c>
     </row>
     <row r="7">
@@ -5973,19 +5973,19 @@
       </c>
       <c r="D7" s="12">
         <f>B7-C7</f>
-        <v/>
+        <v>16.3</v>
       </c>
       <c r="E7" s="14">
         <f>B7*Assumptions!$B$5+28133*Assumptions!$B$4</f>
-        <v/>
+        <v>5218.1577</v>
       </c>
       <c r="F7" s="14">
         <f>C7*Assumptions!$B$5+28133*Assumptions!$B$4</f>
-        <v/>
+        <v>4796.9657</v>
       </c>
       <c r="G7" s="14">
         <f>E7-F7</f>
-        <v/>
+        <v>421.192</v>
       </c>
     </row>
     <row r="8">
@@ -6002,19 +6002,19 @@
       </c>
       <c r="D8" s="12">
         <f>B8-C8</f>
-        <v/>
+        <v>19.6</v>
       </c>
       <c r="E8" s="14">
         <f>B8*Assumptions!$B$5+6245*Assumptions!$B$4</f>
-        <v/>
+        <v>1454.8505</v>
       </c>
       <c r="F8" s="14">
         <f>C8*Assumptions!$B$5+6245*Assumptions!$B$4</f>
-        <v/>
+        <v>948.3865</v>
       </c>
       <c r="G8" s="14">
         <f>E8-F8</f>
-        <v/>
+        <v>506.464</v>
       </c>
     </row>
     <row r="9">
@@ -6031,19 +6031,19 @@
       </c>
       <c r="D9" s="12">
         <f>B9-C9</f>
-        <v/>
+        <v>15.1</v>
       </c>
       <c r="E9" s="14">
         <f>B9*Assumptions!$B$5+4765*Assumptions!$B$4</f>
-        <v/>
+        <v>1213.1985</v>
       </c>
       <c r="F9" s="14">
         <f>C9*Assumptions!$B$5+4765*Assumptions!$B$4</f>
-        <v/>
+        <v>823.0145</v>
       </c>
       <c r="G9" s="14">
         <f>E9-F9</f>
-        <v/>
+        <v>390.184</v>
       </c>
     </row>
     <row r="10">
@@ -6060,19 +6060,19 @@
       </c>
       <c r="D10" s="12">
         <f>B10-C10</f>
-        <v/>
+        <v>15</v>
       </c>
       <c r="E10" s="14">
         <f>B10*Assumptions!$B$5+4316*Assumptions!$B$4</f>
-        <v/>
+        <v>1029.0364</v>
       </c>
       <c r="F10" s="14">
         <f>C10*Assumptions!$B$5+4316*Assumptions!$B$4</f>
-        <v/>
+        <v>641.4364</v>
       </c>
       <c r="G10" s="14">
         <f>E10-F10</f>
-        <v/>
+        <v>387.6</v>
       </c>
     </row>
     <row r="11">
@@ -6089,19 +6089,19 @@
       </c>
       <c r="D11" s="12">
         <f>B11-C11</f>
-        <v/>
+        <v>18.4</v>
       </c>
       <c r="E11" s="14">
         <f>B11*Assumptions!$B$5+3468*Assumptions!$B$4</f>
-        <v/>
+        <v>1004.7612</v>
       </c>
       <c r="F11" s="14">
         <f>C11*Assumptions!$B$5+3468*Assumptions!$B$4</f>
-        <v/>
+        <v>529.3052</v>
       </c>
       <c r="G11" s="14">
         <f>E11-F11</f>
-        <v/>
+        <v>475.456</v>
       </c>
     </row>
     <row r="12">
@@ -6118,19 +6118,19 @@
       </c>
       <c r="D12" s="12">
         <f>B12-C12</f>
-        <v/>
+        <v>11.6</v>
       </c>
       <c r="E12" s="14">
         <f>B12*Assumptions!$B$5+2927*Assumptions!$B$4</f>
-        <v/>
+        <v>761.3003</v>
       </c>
       <c r="F12" s="14">
         <f>C12*Assumptions!$B$5+2927*Assumptions!$B$4</f>
-        <v/>
+        <v>461.5563</v>
       </c>
       <c r="G12" s="14">
         <f>E12-F12</f>
-        <v/>
+        <v>299.744</v>
       </c>
     </row>
     <row r="13">
@@ -6147,19 +6147,19 @@
       </c>
       <c r="D13" s="12">
         <f>B13-C13</f>
-        <v/>
+        <v>12.6</v>
       </c>
       <c r="E13" s="14">
         <f>B13*Assumptions!$B$5+2606*Assumptions!$B$4</f>
-        <v/>
+        <v>764.4614</v>
       </c>
       <c r="F13" s="14">
         <f>C13*Assumptions!$B$5+2606*Assumptions!$B$4</f>
-        <v/>
+        <v>438.8774</v>
       </c>
       <c r="G13" s="14">
         <f>E13-F13</f>
-        <v/>
+        <v>325.584</v>
       </c>
     </row>
     <row r="14">
@@ -6176,19 +6176,19 @@
       </c>
       <c r="D14" s="12">
         <f>B14-C14</f>
-        <v/>
+        <v>24.9</v>
       </c>
       <c r="E14" s="14">
         <f>B14*Assumptions!$B$5+34658*Assumptions!$B$4</f>
-        <v/>
+        <v>6812.5882</v>
       </c>
       <c r="F14" s="14">
         <f>C14*Assumptions!$B$5+34658*Assumptions!$B$4</f>
-        <v/>
+        <v>6169.1722</v>
       </c>
       <c r="G14" s="14">
         <f>E14-F14</f>
-        <v/>
+        <v>643.416</v>
       </c>
     </row>
     <row r="15">
@@ -6205,19 +6205,19 @@
       </c>
       <c r="D15" s="12">
         <f>B15-C15</f>
-        <v/>
+        <v>28</v>
       </c>
       <c r="E15" s="14">
         <f>B15*Assumptions!$B$5+24158*Assumptions!$B$4</f>
-        <v/>
+        <v>4511.1782</v>
       </c>
       <c r="F15" s="14">
         <f>C15*Assumptions!$B$5+24158*Assumptions!$B$4</f>
-        <v/>
+        <v>3787.6582</v>
       </c>
       <c r="G15" s="14">
         <f>E15-F15</f>
-        <v/>
+        <v>723.52</v>
       </c>
     </row>
     <row r="16">
@@ -6235,11 +6235,11 @@
       </c>
       <c r="F16" s="29">
         <f>SUM(F4:F15)</f>
-        <v/>
+        <v>36521.6894</v>
       </c>
       <c r="G16" s="29">
         <f>SUM(G4:G15)</f>
-        <v/>
+        <v>6165.424</v>
       </c>
     </row>
   </sheetData>

</xml_diff>